<commit_message>
changement du libellé de la cellule sur le diamètre
</commit_message>
<xml_diff>
--- a/AutosurveillanceTemplates/Q_DEM.xlsx
+++ b/AutosurveillanceTemplates/Q_DEM.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ndhuy\AppData\Roaming\Microsoft\AddIns\AutosurveillanceTemplates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\autosurveillance_steu_excel\AutosurveillanceTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4257F7C7-8CCE-47B7-9064-C623EEA81B30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6255206-6DA0-42D8-A63E-B482B8F7E3F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-8205" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="777" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1199,9 +1199,6 @@
     <t xml:space="preserve">Fréquence de vérification sur site : </t>
   </si>
   <si>
-    <t xml:space="preserve">Diamètre de la canalisation (mm) : </t>
-  </si>
-  <si>
     <t xml:space="preserve">Longueur droite amont (mm) : </t>
   </si>
   <si>
@@ -2180,6 +2177,9 @@
   </si>
   <si>
     <t>La vanne de prélèvement est-elle asservie au débit, ou au volume écoulé, et assure-t-elle un nombre de prélèvements égal, en moyenne, à au moins à 6 par heure de rejet effectif ? soit 144 prélèvements unitaires par 24h de rejet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diamètre du débitmètre (mm) : </t>
   </si>
 </sst>
 </file>
@@ -4721,6 +4721,234 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="115" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="6" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="33" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="77" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="78" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="16" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="16" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="16" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="16" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="80" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="81" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -4742,23 +4970,6 @@
     <xf numFmtId="0" fontId="35" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="26" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -4771,215 +4982,6 @@
     <xf numFmtId="0" fontId="26" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="18" borderId="77" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="18" borderId="78" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="18" borderId="79" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="80" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="81" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="14" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="14" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="14" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="0" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="0" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="42" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -5007,8 +5009,6 @@
     <xf numFmtId="0" fontId="3" fillId="22" borderId="102" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="33" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Lien hypertexte" xfId="3" builtinId="8"/>
@@ -5476,9 +5476,9 @@
     <col min="1" max="2" width="2.703125" style="63" customWidth="1"/>
     <col min="3" max="18" width="10.703125" style="63"/>
     <col min="19" max="19" width="2.703125" style="63" customWidth="1"/>
-    <col min="20" max="20" width="2.703125" style="279" customWidth="1"/>
-    <col min="21" max="21" width="10.703125" style="280"/>
-    <col min="22" max="28" width="10.703125" style="279"/>
+    <col min="20" max="20" width="2.703125" style="194" customWidth="1"/>
+    <col min="21" max="21" width="10.703125" style="195"/>
+    <col min="22" max="28" width="10.703125" style="194"/>
     <col min="29" max="16384" width="10.703125" style="63"/>
   </cols>
   <sheetData>
@@ -5504,131 +5504,131 @@
     </row>
     <row r="2" spans="2:19" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
       <c r="B2" s="68"/>
-      <c r="C2" s="267" t="s">
-        <v>274</v>
-      </c>
-      <c r="D2" s="268"/>
-      <c r="E2" s="268"/>
-      <c r="F2" s="268"/>
-      <c r="G2" s="268"/>
-      <c r="H2" s="268"/>
-      <c r="I2" s="268"/>
-      <c r="J2" s="268"/>
-      <c r="K2" s="268"/>
-      <c r="L2" s="268"/>
-      <c r="M2" s="268"/>
-      <c r="N2" s="268"/>
-      <c r="O2" s="268"/>
-      <c r="P2" s="268"/>
-      <c r="Q2" s="268"/>
-      <c r="R2" s="269"/>
+      <c r="C2" s="201" t="s">
+        <v>273</v>
+      </c>
+      <c r="D2" s="202"/>
+      <c r="E2" s="202"/>
+      <c r="F2" s="202"/>
+      <c r="G2" s="202"/>
+      <c r="H2" s="202"/>
+      <c r="I2" s="202"/>
+      <c r="J2" s="202"/>
+      <c r="K2" s="202"/>
+      <c r="L2" s="202"/>
+      <c r="M2" s="202"/>
+      <c r="N2" s="202"/>
+      <c r="O2" s="202"/>
+      <c r="P2" s="202"/>
+      <c r="Q2" s="202"/>
+      <c r="R2" s="203"/>
       <c r="S2" s="69"/>
     </row>
     <row r="3" spans="2:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B3" s="70"/>
-      <c r="C3" s="260" t="s">
-        <v>239</v>
-      </c>
-      <c r="D3" s="261"/>
-      <c r="E3" s="262"/>
-      <c r="F3" s="262"/>
-      <c r="G3" s="262"/>
-      <c r="H3" s="261" t="s">
-        <v>219</v>
-      </c>
-      <c r="I3" s="261"/>
-      <c r="J3" s="262"/>
-      <c r="K3" s="262"/>
-      <c r="L3" s="262"/>
-      <c r="M3" s="261" t="s">
-        <v>221</v>
-      </c>
-      <c r="N3" s="261"/>
-      <c r="O3" s="261"/>
-      <c r="P3" s="265"/>
-      <c r="Q3" s="265"/>
-      <c r="R3" s="266"/>
+      <c r="C3" s="196" t="s">
+        <v>238</v>
+      </c>
+      <c r="D3" s="197"/>
+      <c r="E3" s="198"/>
+      <c r="F3" s="198"/>
+      <c r="G3" s="198"/>
+      <c r="H3" s="197" t="s">
+        <v>218</v>
+      </c>
+      <c r="I3" s="197"/>
+      <c r="J3" s="198"/>
+      <c r="K3" s="198"/>
+      <c r="L3" s="198"/>
+      <c r="M3" s="197" t="s">
+        <v>220</v>
+      </c>
+      <c r="N3" s="197"/>
+      <c r="O3" s="197"/>
+      <c r="P3" s="199"/>
+      <c r="Q3" s="199"/>
+      <c r="R3" s="200"/>
       <c r="S3" s="71"/>
     </row>
     <row r="4" spans="2:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B4" s="70"/>
-      <c r="C4" s="260" t="s">
-        <v>216</v>
-      </c>
-      <c r="D4" s="261"/>
-      <c r="E4" s="262"/>
-      <c r="F4" s="262"/>
-      <c r="G4" s="262"/>
-      <c r="H4" s="261" t="s">
+      <c r="C4" s="196" t="s">
+        <v>215</v>
+      </c>
+      <c r="D4" s="197"/>
+      <c r="E4" s="198"/>
+      <c r="F4" s="198"/>
+      <c r="G4" s="198"/>
+      <c r="H4" s="197" t="s">
+        <v>240</v>
+      </c>
+      <c r="I4" s="197"/>
+      <c r="J4" s="198"/>
+      <c r="K4" s="198"/>
+      <c r="L4" s="198"/>
+      <c r="M4" s="197" t="s">
         <v>241</v>
       </c>
-      <c r="I4" s="261"/>
-      <c r="J4" s="262"/>
-      <c r="K4" s="262"/>
-      <c r="L4" s="262"/>
-      <c r="M4" s="261" t="s">
-        <v>242</v>
-      </c>
-      <c r="N4" s="261"/>
-      <c r="O4" s="261"/>
-      <c r="P4" s="265"/>
-      <c r="Q4" s="265"/>
-      <c r="R4" s="266"/>
+      <c r="N4" s="197"/>
+      <c r="O4" s="197"/>
+      <c r="P4" s="199"/>
+      <c r="Q4" s="199"/>
+      <c r="R4" s="200"/>
       <c r="S4" s="71"/>
     </row>
     <row r="5" spans="2:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B5" s="70"/>
-      <c r="C5" s="260" t="s">
-        <v>217</v>
-      </c>
-      <c r="D5" s="261"/>
-      <c r="E5" s="262"/>
-      <c r="F5" s="262"/>
-      <c r="G5" s="262"/>
-      <c r="H5" s="261" t="s">
-        <v>240</v>
-      </c>
-      <c r="I5" s="261"/>
-      <c r="J5" s="262"/>
-      <c r="K5" s="262"/>
-      <c r="L5" s="262"/>
-      <c r="M5" s="261" t="s">
-        <v>222</v>
-      </c>
-      <c r="N5" s="261"/>
-      <c r="O5" s="261"/>
-      <c r="P5" s="263"/>
-      <c r="Q5" s="263"/>
-      <c r="R5" s="264"/>
+      <c r="C5" s="196" t="s">
+        <v>216</v>
+      </c>
+      <c r="D5" s="197"/>
+      <c r="E5" s="198"/>
+      <c r="F5" s="198"/>
+      <c r="G5" s="198"/>
+      <c r="H5" s="197" t="s">
+        <v>239</v>
+      </c>
+      <c r="I5" s="197"/>
+      <c r="J5" s="198"/>
+      <c r="K5" s="198"/>
+      <c r="L5" s="198"/>
+      <c r="M5" s="197" t="s">
+        <v>221</v>
+      </c>
+      <c r="N5" s="197"/>
+      <c r="O5" s="197"/>
+      <c r="P5" s="209"/>
+      <c r="Q5" s="209"/>
+      <c r="R5" s="210"/>
       <c r="S5" s="71"/>
     </row>
     <row r="6" spans="2:19" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B6" s="70"/>
-      <c r="C6" s="255" t="s">
-        <v>218</v>
-      </c>
-      <c r="D6" s="256"/>
-      <c r="E6" s="257"/>
-      <c r="F6" s="257"/>
-      <c r="G6" s="257"/>
-      <c r="H6" s="256" t="s">
-        <v>220</v>
-      </c>
-      <c r="I6" s="256"/>
-      <c r="J6" s="257" t="str">
+      <c r="C6" s="204" t="s">
+        <v>217</v>
+      </c>
+      <c r="D6" s="205"/>
+      <c r="E6" s="206"/>
+      <c r="F6" s="206"/>
+      <c r="G6" s="206"/>
+      <c r="H6" s="205" t="s">
+        <v>219</v>
+      </c>
+      <c r="I6" s="205"/>
+      <c r="J6" s="206" t="str">
         <f>IF(D32&lt;&gt;"",D32,"")</f>
         <v/>
       </c>
-      <c r="K6" s="257"/>
-      <c r="L6" s="257"/>
-      <c r="M6" s="256" t="s">
-        <v>243</v>
-      </c>
-      <c r="N6" s="256"/>
-      <c r="O6" s="256"/>
-      <c r="P6" s="258"/>
-      <c r="Q6" s="258"/>
-      <c r="R6" s="259"/>
+      <c r="K6" s="206"/>
+      <c r="L6" s="206"/>
+      <c r="M6" s="205" t="s">
+        <v>242</v>
+      </c>
+      <c r="N6" s="205"/>
+      <c r="O6" s="205"/>
+      <c r="P6" s="207"/>
+      <c r="Q6" s="207"/>
+      <c r="R6" s="208"/>
       <c r="S6" s="71"/>
     </row>
     <row r="7" spans="2:19" ht="9.9499999999999993" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
@@ -5653,24 +5653,24 @@
     </row>
     <row r="8" spans="2:19" ht="20.100000000000001" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B8" s="72"/>
-      <c r="C8" s="209" t="s">
+      <c r="C8" s="211" t="s">
         <v>190</v>
       </c>
-      <c r="D8" s="210"/>
-      <c r="E8" s="210"/>
-      <c r="F8" s="210"/>
-      <c r="G8" s="210"/>
-      <c r="H8" s="210"/>
-      <c r="I8" s="210"/>
-      <c r="J8" s="210"/>
-      <c r="K8" s="210"/>
-      <c r="L8" s="210"/>
-      <c r="M8" s="210"/>
-      <c r="N8" s="210"/>
-      <c r="O8" s="210"/>
-      <c r="P8" s="210"/>
-      <c r="Q8" s="210"/>
-      <c r="R8" s="211"/>
+      <c r="D8" s="212"/>
+      <c r="E8" s="212"/>
+      <c r="F8" s="212"/>
+      <c r="G8" s="212"/>
+      <c r="H8" s="212"/>
+      <c r="I8" s="212"/>
+      <c r="J8" s="212"/>
+      <c r="K8" s="212"/>
+      <c r="L8" s="212"/>
+      <c r="M8" s="212"/>
+      <c r="N8" s="212"/>
+      <c r="O8" s="212"/>
+      <c r="P8" s="212"/>
+      <c r="Q8" s="212"/>
+      <c r="R8" s="213"/>
       <c r="S8" s="74"/>
     </row>
     <row r="9" spans="2:19" ht="20.100000000000001" customHeight="1" outlineLevel="1" thickTop="1" x14ac:dyDescent="0.4">
@@ -5696,142 +5696,142 @@
     <row r="10" spans="2:19" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B10" s="72"/>
       <c r="C10" s="91"/>
-      <c r="D10" s="239" t="s">
+      <c r="D10" s="220" t="s">
         <v>192</v>
       </c>
-      <c r="E10" s="240"/>
-      <c r="F10" s="240"/>
-      <c r="G10" s="240"/>
-      <c r="H10" s="240"/>
-      <c r="I10" s="240"/>
-      <c r="J10" s="240"/>
-      <c r="K10" s="240"/>
-      <c r="L10" s="240"/>
-      <c r="M10" s="240"/>
-      <c r="N10" s="240"/>
-      <c r="O10" s="240"/>
-      <c r="P10" s="240"/>
-      <c r="Q10" s="245"/>
+      <c r="E10" s="221"/>
+      <c r="F10" s="221"/>
+      <c r="G10" s="221"/>
+      <c r="H10" s="221"/>
+      <c r="I10" s="221"/>
+      <c r="J10" s="221"/>
+      <c r="K10" s="221"/>
+      <c r="L10" s="221"/>
+      <c r="M10" s="221"/>
+      <c r="N10" s="221"/>
+      <c r="O10" s="221"/>
+      <c r="P10" s="221"/>
+      <c r="Q10" s="222"/>
       <c r="R10" s="92"/>
       <c r="S10" s="74"/>
     </row>
     <row r="11" spans="2:19" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B11" s="72"/>
       <c r="C11" s="91"/>
-      <c r="D11" s="233" t="s">
-        <v>223</v>
-      </c>
-      <c r="E11" s="234"/>
-      <c r="F11" s="235"/>
-      <c r="G11" s="242"/>
-      <c r="H11" s="243"/>
-      <c r="I11" s="243"/>
-      <c r="J11" s="244"/>
-      <c r="K11" s="233" t="s">
+      <c r="D11" s="223" t="s">
+        <v>222</v>
+      </c>
+      <c r="E11" s="224"/>
+      <c r="F11" s="225"/>
+      <c r="G11" s="226"/>
+      <c r="H11" s="227"/>
+      <c r="I11" s="227"/>
+      <c r="J11" s="228"/>
+      <c r="K11" s="223" t="s">
         <v>193</v>
       </c>
-      <c r="L11" s="234"/>
-      <c r="M11" s="235"/>
-      <c r="N11" s="236"/>
-      <c r="O11" s="237"/>
-      <c r="P11" s="237"/>
-      <c r="Q11" s="238"/>
+      <c r="L11" s="224"/>
+      <c r="M11" s="225"/>
+      <c r="N11" s="229"/>
+      <c r="O11" s="230"/>
+      <c r="P11" s="230"/>
+      <c r="Q11" s="231"/>
       <c r="R11" s="92"/>
       <c r="S11" s="74"/>
     </row>
     <row r="12" spans="2:19" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B12" s="72"/>
       <c r="C12" s="91"/>
-      <c r="D12" s="233" t="s">
+      <c r="D12" s="223" t="s">
         <v>176</v>
       </c>
-      <c r="E12" s="234"/>
-      <c r="F12" s="235"/>
-      <c r="G12" s="242"/>
-      <c r="H12" s="243"/>
-      <c r="I12" s="243"/>
-      <c r="J12" s="244"/>
-      <c r="K12" s="233" t="s">
-        <v>235</v>
-      </c>
-      <c r="L12" s="234"/>
-      <c r="M12" s="235"/>
-      <c r="N12" s="252"/>
-      <c r="O12" s="253"/>
-      <c r="P12" s="253"/>
-      <c r="Q12" s="254"/>
+      <c r="E12" s="224"/>
+      <c r="F12" s="225"/>
+      <c r="G12" s="226"/>
+      <c r="H12" s="227"/>
+      <c r="I12" s="227"/>
+      <c r="J12" s="228"/>
+      <c r="K12" s="223" t="s">
+        <v>234</v>
+      </c>
+      <c r="L12" s="224"/>
+      <c r="M12" s="225"/>
+      <c r="N12" s="232"/>
+      <c r="O12" s="233"/>
+      <c r="P12" s="233"/>
+      <c r="Q12" s="234"/>
       <c r="R12" s="92"/>
       <c r="S12" s="74"/>
     </row>
     <row r="13" spans="2:19" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B13" s="72"/>
       <c r="C13" s="91"/>
-      <c r="D13" s="233" t="s">
-        <v>233</v>
-      </c>
-      <c r="E13" s="234"/>
-      <c r="F13" s="235"/>
-      <c r="G13" s="242"/>
-      <c r="H13" s="243"/>
-      <c r="I13" s="243"/>
-      <c r="J13" s="244"/>
-      <c r="K13" s="233" t="s">
-        <v>194</v>
-      </c>
-      <c r="L13" s="234"/>
-      <c r="M13" s="235"/>
-      <c r="N13" s="242"/>
-      <c r="O13" s="243"/>
-      <c r="P13" s="243"/>
-      <c r="Q13" s="244"/>
+      <c r="D13" s="223" t="s">
+        <v>232</v>
+      </c>
+      <c r="E13" s="224"/>
+      <c r="F13" s="225"/>
+      <c r="G13" s="226"/>
+      <c r="H13" s="227"/>
+      <c r="I13" s="227"/>
+      <c r="J13" s="228"/>
+      <c r="K13" s="223" t="s">
+        <v>341</v>
+      </c>
+      <c r="L13" s="224"/>
+      <c r="M13" s="225"/>
+      <c r="N13" s="226"/>
+      <c r="O13" s="227"/>
+      <c r="P13" s="227"/>
+      <c r="Q13" s="228"/>
       <c r="R13" s="92"/>
       <c r="S13" s="74"/>
     </row>
     <row r="14" spans="2:19" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B14" s="72"/>
       <c r="C14" s="91"/>
-      <c r="D14" s="233" t="s">
-        <v>234</v>
-      </c>
-      <c r="E14" s="234"/>
-      <c r="F14" s="235"/>
-      <c r="G14" s="242"/>
-      <c r="H14" s="243"/>
-      <c r="I14" s="243"/>
-      <c r="J14" s="244"/>
-      <c r="K14" s="233" t="s">
-        <v>195</v>
-      </c>
-      <c r="L14" s="234"/>
-      <c r="M14" s="235"/>
-      <c r="N14" s="242"/>
-      <c r="O14" s="243"/>
-      <c r="P14" s="243"/>
-      <c r="Q14" s="244"/>
+      <c r="D14" s="223" t="s">
+        <v>233</v>
+      </c>
+      <c r="E14" s="224"/>
+      <c r="F14" s="225"/>
+      <c r="G14" s="226"/>
+      <c r="H14" s="227"/>
+      <c r="I14" s="227"/>
+      <c r="J14" s="228"/>
+      <c r="K14" s="223" t="s">
+        <v>194</v>
+      </c>
+      <c r="L14" s="224"/>
+      <c r="M14" s="225"/>
+      <c r="N14" s="226"/>
+      <c r="O14" s="227"/>
+      <c r="P14" s="227"/>
+      <c r="Q14" s="228"/>
       <c r="R14" s="92"/>
       <c r="S14" s="74"/>
     </row>
     <row r="15" spans="2:19" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B15" s="72"/>
       <c r="C15" s="91"/>
-      <c r="D15" s="233" t="s">
-        <v>215</v>
-      </c>
-      <c r="E15" s="234"/>
-      <c r="F15" s="235"/>
-      <c r="G15" s="242"/>
-      <c r="H15" s="243"/>
-      <c r="I15" s="243"/>
-      <c r="J15" s="244"/>
-      <c r="K15" s="233" t="s">
-        <v>196</v>
-      </c>
-      <c r="L15" s="234"/>
-      <c r="M15" s="235"/>
-      <c r="N15" s="242"/>
-      <c r="O15" s="243"/>
-      <c r="P15" s="243"/>
-      <c r="Q15" s="244"/>
+      <c r="D15" s="223" t="s">
+        <v>214</v>
+      </c>
+      <c r="E15" s="224"/>
+      <c r="F15" s="225"/>
+      <c r="G15" s="226"/>
+      <c r="H15" s="227"/>
+      <c r="I15" s="227"/>
+      <c r="J15" s="228"/>
+      <c r="K15" s="223" t="s">
+        <v>195</v>
+      </c>
+      <c r="L15" s="224"/>
+      <c r="M15" s="225"/>
+      <c r="N15" s="226"/>
+      <c r="O15" s="227"/>
+      <c r="P15" s="227"/>
+      <c r="Q15" s="228"/>
       <c r="R15" s="92"/>
       <c r="S15" s="74"/>
     </row>
@@ -5858,142 +5858,142 @@
     <row r="17" spans="2:24" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B17" s="72"/>
       <c r="C17" s="91"/>
-      <c r="D17" s="239" t="s">
-        <v>206</v>
-      </c>
-      <c r="E17" s="240"/>
-      <c r="F17" s="240"/>
-      <c r="G17" s="240"/>
-      <c r="H17" s="240"/>
-      <c r="I17" s="240"/>
-      <c r="J17" s="240"/>
-      <c r="K17" s="240"/>
-      <c r="L17" s="240"/>
-      <c r="M17" s="240"/>
-      <c r="N17" s="240"/>
-      <c r="O17" s="240"/>
-      <c r="P17" s="240"/>
-      <c r="Q17" s="245"/>
+      <c r="D17" s="220" t="s">
+        <v>205</v>
+      </c>
+      <c r="E17" s="221"/>
+      <c r="F17" s="221"/>
+      <c r="G17" s="221"/>
+      <c r="H17" s="221"/>
+      <c r="I17" s="221"/>
+      <c r="J17" s="221"/>
+      <c r="K17" s="221"/>
+      <c r="L17" s="221"/>
+      <c r="M17" s="221"/>
+      <c r="N17" s="221"/>
+      <c r="O17" s="221"/>
+      <c r="P17" s="221"/>
+      <c r="Q17" s="222"/>
       <c r="R17" s="92"/>
       <c r="S17" s="74"/>
     </row>
     <row r="18" spans="2:24" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B18" s="72"/>
       <c r="C18" s="91"/>
-      <c r="D18" s="233" t="s">
-        <v>224</v>
-      </c>
-      <c r="E18" s="234"/>
-      <c r="F18" s="235"/>
-      <c r="G18" s="236"/>
-      <c r="H18" s="237"/>
-      <c r="I18" s="237"/>
-      <c r="J18" s="238"/>
-      <c r="K18" s="233" t="s">
-        <v>229</v>
-      </c>
-      <c r="L18" s="234"/>
-      <c r="M18" s="235"/>
-      <c r="N18" s="242"/>
-      <c r="O18" s="243"/>
-      <c r="P18" s="243"/>
-      <c r="Q18" s="244"/>
+      <c r="D18" s="223" t="s">
+        <v>223</v>
+      </c>
+      <c r="E18" s="224"/>
+      <c r="F18" s="225"/>
+      <c r="G18" s="229"/>
+      <c r="H18" s="230"/>
+      <c r="I18" s="230"/>
+      <c r="J18" s="231"/>
+      <c r="K18" s="223" t="s">
+        <v>228</v>
+      </c>
+      <c r="L18" s="224"/>
+      <c r="M18" s="225"/>
+      <c r="N18" s="226"/>
+      <c r="O18" s="227"/>
+      <c r="P18" s="227"/>
+      <c r="Q18" s="228"/>
       <c r="R18" s="92"/>
       <c r="S18" s="74"/>
     </row>
     <row r="19" spans="2:24" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B19" s="72"/>
       <c r="C19" s="91"/>
-      <c r="D19" s="233" t="s">
-        <v>225</v>
-      </c>
-      <c r="E19" s="234"/>
-      <c r="F19" s="235"/>
-      <c r="G19" s="236"/>
-      <c r="H19" s="237"/>
-      <c r="I19" s="237"/>
-      <c r="J19" s="238"/>
-      <c r="K19" s="233" t="s">
-        <v>244</v>
-      </c>
-      <c r="L19" s="234"/>
-      <c r="M19" s="235"/>
-      <c r="N19" s="242"/>
-      <c r="O19" s="243"/>
-      <c r="P19" s="243"/>
-      <c r="Q19" s="244"/>
+      <c r="D19" s="223" t="s">
+        <v>224</v>
+      </c>
+      <c r="E19" s="224"/>
+      <c r="F19" s="225"/>
+      <c r="G19" s="229"/>
+      <c r="H19" s="230"/>
+      <c r="I19" s="230"/>
+      <c r="J19" s="231"/>
+      <c r="K19" s="223" t="s">
+        <v>243</v>
+      </c>
+      <c r="L19" s="224"/>
+      <c r="M19" s="225"/>
+      <c r="N19" s="226"/>
+      <c r="O19" s="227"/>
+      <c r="P19" s="227"/>
+      <c r="Q19" s="228"/>
       <c r="R19" s="92"/>
       <c r="S19" s="74"/>
     </row>
     <row r="20" spans="2:24" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B20" s="72"/>
       <c r="C20" s="91"/>
-      <c r="D20" s="233" t="s">
-        <v>226</v>
-      </c>
-      <c r="E20" s="234"/>
-      <c r="F20" s="235"/>
-      <c r="G20" s="236"/>
-      <c r="H20" s="237"/>
-      <c r="I20" s="237"/>
-      <c r="J20" s="238"/>
-      <c r="K20" s="233" t="s">
-        <v>230</v>
-      </c>
-      <c r="L20" s="234"/>
-      <c r="M20" s="235"/>
-      <c r="N20" s="242"/>
-      <c r="O20" s="243"/>
-      <c r="P20" s="243"/>
-      <c r="Q20" s="244"/>
+      <c r="D20" s="223" t="s">
+        <v>225</v>
+      </c>
+      <c r="E20" s="224"/>
+      <c r="F20" s="225"/>
+      <c r="G20" s="229"/>
+      <c r="H20" s="230"/>
+      <c r="I20" s="230"/>
+      <c r="J20" s="231"/>
+      <c r="K20" s="223" t="s">
+        <v>229</v>
+      </c>
+      <c r="L20" s="224"/>
+      <c r="M20" s="225"/>
+      <c r="N20" s="226"/>
+      <c r="O20" s="227"/>
+      <c r="P20" s="227"/>
+      <c r="Q20" s="228"/>
       <c r="R20" s="92"/>
       <c r="S20" s="74"/>
     </row>
     <row r="21" spans="2:24" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B21" s="72"/>
       <c r="C21" s="91"/>
-      <c r="D21" s="233" t="s">
-        <v>227</v>
-      </c>
-      <c r="E21" s="234"/>
-      <c r="F21" s="235"/>
-      <c r="G21" s="236"/>
-      <c r="H21" s="237"/>
-      <c r="I21" s="237"/>
-      <c r="J21" s="238"/>
-      <c r="K21" s="233" t="s">
-        <v>231</v>
-      </c>
-      <c r="L21" s="234"/>
-      <c r="M21" s="235"/>
-      <c r="N21" s="236"/>
-      <c r="O21" s="237"/>
-      <c r="P21" s="237"/>
-      <c r="Q21" s="238"/>
+      <c r="D21" s="223" t="s">
+        <v>226</v>
+      </c>
+      <c r="E21" s="224"/>
+      <c r="F21" s="225"/>
+      <c r="G21" s="229"/>
+      <c r="H21" s="230"/>
+      <c r="I21" s="230"/>
+      <c r="J21" s="231"/>
+      <c r="K21" s="223" t="s">
+        <v>230</v>
+      </c>
+      <c r="L21" s="224"/>
+      <c r="M21" s="225"/>
+      <c r="N21" s="229"/>
+      <c r="O21" s="230"/>
+      <c r="P21" s="230"/>
+      <c r="Q21" s="231"/>
       <c r="R21" s="92"/>
       <c r="S21" s="74"/>
     </row>
     <row r="22" spans="2:24" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B22" s="72"/>
       <c r="C22" s="91"/>
-      <c r="D22" s="233" t="s">
-        <v>228</v>
-      </c>
-      <c r="E22" s="234"/>
-      <c r="F22" s="235"/>
-      <c r="G22" s="236"/>
-      <c r="H22" s="237"/>
-      <c r="I22" s="237"/>
-      <c r="J22" s="238"/>
-      <c r="K22" s="233" t="s">
-        <v>232</v>
-      </c>
-      <c r="L22" s="234"/>
-      <c r="M22" s="235"/>
-      <c r="N22" s="236"/>
-      <c r="O22" s="237"/>
-      <c r="P22" s="237"/>
-      <c r="Q22" s="238"/>
+      <c r="D22" s="223" t="s">
+        <v>227</v>
+      </c>
+      <c r="E22" s="224"/>
+      <c r="F22" s="225"/>
+      <c r="G22" s="229"/>
+      <c r="H22" s="230"/>
+      <c r="I22" s="230"/>
+      <c r="J22" s="231"/>
+      <c r="K22" s="223" t="s">
+        <v>231</v>
+      </c>
+      <c r="L22" s="224"/>
+      <c r="M22" s="225"/>
+      <c r="N22" s="229"/>
+      <c r="O22" s="230"/>
+      <c r="P22" s="230"/>
+      <c r="Q22" s="231"/>
       <c r="R22" s="92"/>
       <c r="S22" s="74"/>
     </row>
@@ -6020,22 +6020,22 @@
     <row r="24" spans="2:24" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B24" s="72"/>
       <c r="C24" s="91"/>
-      <c r="D24" s="239" t="s">
+      <c r="D24" s="220" t="s">
         <v>81</v>
       </c>
-      <c r="E24" s="240"/>
-      <c r="F24" s="240"/>
-      <c r="G24" s="240"/>
-      <c r="H24" s="240"/>
-      <c r="I24" s="240"/>
-      <c r="J24" s="240"/>
-      <c r="K24" s="240"/>
-      <c r="L24" s="240"/>
-      <c r="M24" s="240"/>
-      <c r="N24" s="241" t="s">
-        <v>214</v>
-      </c>
-      <c r="O24" s="241"/>
+      <c r="E24" s="221"/>
+      <c r="F24" s="221"/>
+      <c r="G24" s="221"/>
+      <c r="H24" s="221"/>
+      <c r="I24" s="221"/>
+      <c r="J24" s="221"/>
+      <c r="K24" s="221"/>
+      <c r="L24" s="221"/>
+      <c r="M24" s="221"/>
+      <c r="N24" s="248" t="s">
+        <v>213</v>
+      </c>
+      <c r="O24" s="248"/>
       <c r="P24" s="100"/>
       <c r="Q24" s="64"/>
       <c r="R24" s="92"/>
@@ -6044,27 +6044,27 @@
     <row r="25" spans="2:24" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B25" s="72"/>
       <c r="C25" s="91"/>
-      <c r="D25" s="227" t="s">
-        <v>204</v>
-      </c>
-      <c r="E25" s="228"/>
-      <c r="F25" s="229"/>
-      <c r="G25" s="222" t="s">
+      <c r="D25" s="242" t="s">
+        <v>203</v>
+      </c>
+      <c r="E25" s="243"/>
+      <c r="F25" s="244"/>
+      <c r="G25" s="235" t="s">
+        <v>197</v>
+      </c>
+      <c r="H25" s="236"/>
+      <c r="I25" s="236"/>
+      <c r="J25" s="237"/>
+      <c r="K25" s="245" t="s">
         <v>198</v>
       </c>
-      <c r="H25" s="223"/>
-      <c r="I25" s="223"/>
-      <c r="J25" s="224"/>
-      <c r="K25" s="230" t="s">
+      <c r="L25" s="246"/>
+      <c r="M25" s="247"/>
+      <c r="N25" s="245" t="s">
         <v>199</v>
       </c>
-      <c r="L25" s="231"/>
-      <c r="M25" s="232"/>
-      <c r="N25" s="230" t="s">
-        <v>200</v>
-      </c>
-      <c r="O25" s="231"/>
-      <c r="P25" s="232"/>
+      <c r="O25" s="246"/>
+      <c r="P25" s="247"/>
       <c r="Q25" s="64"/>
       <c r="R25" s="92"/>
       <c r="S25" s="74"/>
@@ -6072,38 +6072,38 @@
     <row r="26" spans="2:24" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B26" s="72"/>
       <c r="C26" s="91"/>
-      <c r="D26" s="218" t="s">
+      <c r="D26" s="260" t="s">
+        <v>235</v>
+      </c>
+      <c r="E26" s="261"/>
+      <c r="F26" s="88" t="s">
+        <v>200</v>
+      </c>
+      <c r="G26" s="238" t="s">
+        <v>244</v>
+      </c>
+      <c r="H26" s="239"/>
+      <c r="I26" s="256" t="s">
         <v>236</v>
       </c>
-      <c r="E26" s="219"/>
-      <c r="F26" s="88" t="s">
+      <c r="J26" s="257"/>
+      <c r="K26" s="81" t="s">
         <v>201</v>
       </c>
-      <c r="G26" s="225" t="s">
-        <v>245</v>
-      </c>
-      <c r="H26" s="226"/>
-      <c r="I26" s="214" t="s">
+      <c r="L26" s="82" t="s">
         <v>237</v>
       </c>
-      <c r="J26" s="215"/>
-      <c r="K26" s="81" t="s">
+      <c r="M26" s="83" t="s">
         <v>202</v>
       </c>
-      <c r="L26" s="82" t="s">
-        <v>238</v>
-      </c>
-      <c r="M26" s="83" t="s">
-        <v>203</v>
-      </c>
       <c r="N26" s="81" t="s">
+        <v>201</v>
+      </c>
+      <c r="O26" s="82" t="s">
+        <v>237</v>
+      </c>
+      <c r="P26" s="83" t="s">
         <v>202</v>
-      </c>
-      <c r="O26" s="82" t="s">
-        <v>238</v>
-      </c>
-      <c r="P26" s="83" t="s">
-        <v>203</v>
       </c>
       <c r="Q26" s="64"/>
       <c r="R26" s="92"/>
@@ -6112,16 +6112,16 @@
     <row r="27" spans="2:24" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B27" s="72"/>
       <c r="C27" s="91"/>
-      <c r="D27" s="220"/>
-      <c r="E27" s="221"/>
+      <c r="D27" s="240"/>
+      <c r="E27" s="241"/>
       <c r="F27" s="84" t="str">
         <f>IF(D27="","",IF(D32="Débitmètre électromagnétique (Boue/MDV)",0.1,IF(D27&gt;50,0.05,0.1)))</f>
         <v/>
       </c>
-      <c r="G27" s="220"/>
-      <c r="H27" s="221"/>
-      <c r="I27" s="216"/>
-      <c r="J27" s="217"/>
+      <c r="G27" s="240"/>
+      <c r="H27" s="241"/>
+      <c r="I27" s="258"/>
+      <c r="J27" s="259"/>
       <c r="K27" s="85" t="str">
         <f>IF(AND(D27&lt;&gt;"",G27&lt;&gt;""),(D27+G27)/2,"")</f>
         <v/>
@@ -6149,7 +6149,7 @@
       <c r="Q27" s="64"/>
       <c r="R27" s="92"/>
       <c r="S27" s="74"/>
-      <c r="U27" s="280" t="str">
+      <c r="U27" s="195" t="str">
         <f>IF(OR(M27&lt;&gt;"",P27&lt;&gt;""),IF(OR(ABS(M27)&gt;0.1,ABS(P27)&gt;0.1),"Non validé (&gt;10%)",IF(AND(ABS(M27)&lt;=0.05,ABS(P27)&lt;=0.05),"Validé","Entre 5 et 10%")),"Non contrôlé")</f>
         <v>Non contrôlé</v>
       </c>
@@ -6196,24 +6196,24 @@
     </row>
     <row r="30" spans="2:24" ht="20.100000000000001" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B30" s="72"/>
-      <c r="C30" s="209" t="s">
-        <v>246</v>
-      </c>
-      <c r="D30" s="210"/>
-      <c r="E30" s="210"/>
-      <c r="F30" s="210"/>
-      <c r="G30" s="210"/>
-      <c r="H30" s="210"/>
-      <c r="I30" s="210"/>
-      <c r="J30" s="210"/>
-      <c r="K30" s="210"/>
-      <c r="L30" s="210"/>
-      <c r="M30" s="210"/>
-      <c r="N30" s="210"/>
-      <c r="O30" s="210"/>
-      <c r="P30" s="210"/>
-      <c r="Q30" s="210"/>
-      <c r="R30" s="211"/>
+      <c r="C30" s="211" t="s">
+        <v>245</v>
+      </c>
+      <c r="D30" s="212"/>
+      <c r="E30" s="212"/>
+      <c r="F30" s="212"/>
+      <c r="G30" s="212"/>
+      <c r="H30" s="212"/>
+      <c r="I30" s="212"/>
+      <c r="J30" s="212"/>
+      <c r="K30" s="212"/>
+      <c r="L30" s="212"/>
+      <c r="M30" s="212"/>
+      <c r="N30" s="212"/>
+      <c r="O30" s="212"/>
+      <c r="P30" s="212"/>
+      <c r="Q30" s="212"/>
+      <c r="R30" s="213"/>
       <c r="S30" s="74"/>
     </row>
     <row r="31" spans="2:24" ht="20.100000000000001" customHeight="1" outlineLevel="1" thickTop="1" x14ac:dyDescent="0.4">
@@ -6239,55 +6239,55 @@
     <row r="32" spans="2:24" ht="30" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B32" s="72"/>
       <c r="C32" s="91"/>
-      <c r="D32" s="212"/>
-      <c r="E32" s="212"/>
-      <c r="F32" s="212"/>
-      <c r="G32" s="212"/>
-      <c r="H32" s="212"/>
-      <c r="I32" s="212"/>
-      <c r="J32" s="212"/>
-      <c r="K32" s="212"/>
-      <c r="L32" s="212"/>
-      <c r="M32" s="212"/>
-      <c r="N32" s="212"/>
-      <c r="O32" s="212"/>
-      <c r="P32" s="212"/>
-      <c r="Q32" s="212"/>
+      <c r="D32" s="249"/>
+      <c r="E32" s="249"/>
+      <c r="F32" s="249"/>
+      <c r="G32" s="249"/>
+      <c r="H32" s="249"/>
+      <c r="I32" s="249"/>
+      <c r="J32" s="249"/>
+      <c r="K32" s="249"/>
+      <c r="L32" s="249"/>
+      <c r="M32" s="249"/>
+      <c r="N32" s="249"/>
+      <c r="O32" s="249"/>
+      <c r="P32" s="249"/>
+      <c r="Q32" s="249"/>
       <c r="R32" s="92"/>
       <c r="S32" s="74"/>
-      <c r="W32" s="280"/>
-      <c r="X32" s="280"/>
+      <c r="W32" s="195"/>
+      <c r="X32" s="195"/>
     </row>
     <row r="33" spans="2:21" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B33" s="72"/>
       <c r="C33" s="91"/>
-      <c r="D33" s="213" t="s">
+      <c r="D33" s="250" t="s">
         <v>4</v>
       </c>
-      <c r="E33" s="213"/>
-      <c r="F33" s="213"/>
-      <c r="G33" s="213"/>
-      <c r="H33" s="213"/>
-      <c r="I33" s="213"/>
-      <c r="J33" s="213" t="s">
+      <c r="E33" s="250"/>
+      <c r="F33" s="250"/>
+      <c r="G33" s="250"/>
+      <c r="H33" s="250"/>
+      <c r="I33" s="250"/>
+      <c r="J33" s="250" t="s">
         <v>175</v>
       </c>
-      <c r="K33" s="213"/>
-      <c r="L33" s="213"/>
-      <c r="M33" s="213"/>
-      <c r="N33" s="213" t="s">
+      <c r="K33" s="250"/>
+      <c r="L33" s="250"/>
+      <c r="M33" s="250"/>
+      <c r="N33" s="250" t="s">
         <v>75</v>
       </c>
-      <c r="O33" s="213"/>
+      <c r="O33" s="250"/>
       <c r="P33" s="89" t="s">
         <v>189</v>
       </c>
       <c r="Q33" s="89" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="R33" s="92"/>
       <c r="S33" s="74"/>
-      <c r="U33" s="280" t="s">
+      <c r="U33" s="195" t="s">
         <v>5</v>
       </c>
     </row>
@@ -6297,23 +6297,23 @@
       <c r="D34" s="90">
         <v>1</v>
       </c>
-      <c r="E34" s="200" t="str">
+      <c r="E34" s="251" t="str">
         <f>IFERROR(HLOOKUP($D$32,Critères!$B$3:$BE$16,D34+2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="F34" s="201"/>
-      <c r="G34" s="201"/>
-      <c r="H34" s="201"/>
-      <c r="I34" s="202"/>
-      <c r="J34" s="200" t="str">
+      <c r="F34" s="252"/>
+      <c r="G34" s="252"/>
+      <c r="H34" s="252"/>
+      <c r="I34" s="253"/>
+      <c r="J34" s="251" t="str">
         <f>IFERROR(IF(INDEX(Critères!$B$3:$BE$16, D34+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)="", "", INDEX(Critères!$B$3:$BE$16, D34+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)), "")</f>
         <v/>
       </c>
-      <c r="K34" s="201"/>
-      <c r="L34" s="201"/>
-      <c r="M34" s="202"/>
-      <c r="N34" s="203"/>
-      <c r="O34" s="204"/>
+      <c r="K34" s="252"/>
+      <c r="L34" s="252"/>
+      <c r="M34" s="253"/>
+      <c r="N34" s="254"/>
+      <c r="O34" s="255"/>
       <c r="P34" s="87">
         <f>IF(OR(N34="Validé",N34="Réserve",N34="Oui",N34="Entre 5 et 10%"),Q34,0)</f>
         <v>0</v>
@@ -6324,7 +6324,7 @@
       </c>
       <c r="R34" s="92"/>
       <c r="S34" s="74"/>
-      <c r="U34" s="280" t="s">
+      <c r="U34" s="195" t="s">
         <v>40</v>
       </c>
     </row>
@@ -6334,23 +6334,23 @@
       <c r="D35" s="90">
         <v>2</v>
       </c>
-      <c r="E35" s="200" t="str">
+      <c r="E35" s="251" t="str">
         <f>IFERROR(HLOOKUP($D$32,Critères!$B$3:$BE$16,D35+2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="F35" s="201"/>
-      <c r="G35" s="201"/>
-      <c r="H35" s="201"/>
-      <c r="I35" s="202"/>
-      <c r="J35" s="200" t="str">
+      <c r="F35" s="252"/>
+      <c r="G35" s="252"/>
+      <c r="H35" s="252"/>
+      <c r="I35" s="253"/>
+      <c r="J35" s="251" t="str">
         <f>IFERROR(IF(INDEX(Critères!$B$3:$BE$16, D35+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)="", "", INDEX(Critères!$B$3:$BE$16, D35+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)), "")</f>
         <v/>
       </c>
-      <c r="K35" s="201"/>
-      <c r="L35" s="201"/>
-      <c r="M35" s="202"/>
-      <c r="N35" s="203"/>
-      <c r="O35" s="204"/>
+      <c r="K35" s="252"/>
+      <c r="L35" s="252"/>
+      <c r="M35" s="253"/>
+      <c r="N35" s="254"/>
+      <c r="O35" s="255"/>
       <c r="P35" s="87">
         <f t="shared" ref="P35:P42" si="0">IF(OR(N35="Validé",N35="Réserve"),Q35,0)</f>
         <v>0</v>
@@ -6361,7 +6361,7 @@
       </c>
       <c r="R35" s="92"/>
       <c r="S35" s="74"/>
-      <c r="U35" s="280" t="s">
+      <c r="U35" s="195" t="s">
         <v>40</v>
       </c>
     </row>
@@ -6371,23 +6371,23 @@
       <c r="D36" s="90">
         <v>3</v>
       </c>
-      <c r="E36" s="200" t="str">
+      <c r="E36" s="251" t="str">
         <f>IFERROR(HLOOKUP($D$32,Critères!$B$3:$BE$16,D36+2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="F36" s="201"/>
-      <c r="G36" s="201"/>
-      <c r="H36" s="201"/>
-      <c r="I36" s="202"/>
-      <c r="J36" s="200" t="str">
+      <c r="F36" s="252"/>
+      <c r="G36" s="252"/>
+      <c r="H36" s="252"/>
+      <c r="I36" s="253"/>
+      <c r="J36" s="251" t="str">
         <f>IFERROR(IF(INDEX(Critères!$B$3:$BE$16, D36+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)="", "", INDEX(Critères!$B$3:$BE$16, D36+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)), "")</f>
         <v/>
       </c>
-      <c r="K36" s="201"/>
-      <c r="L36" s="201"/>
-      <c r="M36" s="202"/>
-      <c r="N36" s="203"/>
-      <c r="O36" s="204"/>
+      <c r="K36" s="252"/>
+      <c r="L36" s="252"/>
+      <c r="M36" s="253"/>
+      <c r="N36" s="254"/>
+      <c r="O36" s="255"/>
       <c r="P36" s="87">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -6398,7 +6398,7 @@
       </c>
       <c r="R36" s="92"/>
       <c r="S36" s="74"/>
-      <c r="U36" s="280" t="s">
+      <c r="U36" s="195" t="s">
         <v>40</v>
       </c>
     </row>
@@ -6408,26 +6408,26 @@
       <c r="D37" s="90">
         <v>4</v>
       </c>
-      <c r="E37" s="200" t="str">
+      <c r="E37" s="251" t="str">
         <f>IFERROR(HLOOKUP($D$32,Critères!$B$3:$BE$16,D37+2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="F37" s="201"/>
-      <c r="G37" s="201"/>
-      <c r="H37" s="201"/>
-      <c r="I37" s="202"/>
-      <c r="J37" s="200" t="str">
+      <c r="F37" s="252"/>
+      <c r="G37" s="252"/>
+      <c r="H37" s="252"/>
+      <c r="I37" s="253"/>
+      <c r="J37" s="251" t="str">
         <f>IFERROR(IF(INDEX(Critères!$B$3:$BE$16, D37+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)="", "", INDEX(Critères!$B$3:$BE$16, D37+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)), "")</f>
         <v/>
       </c>
-      <c r="K37" s="201"/>
-      <c r="L37" s="201"/>
-      <c r="M37" s="202"/>
-      <c r="N37" s="203" t="str">
+      <c r="K37" s="252"/>
+      <c r="L37" s="252"/>
+      <c r="M37" s="253"/>
+      <c r="N37" s="254" t="str">
         <f>IF(OR(D32 = Critères!B3, D32 = Critères!F3),U27,"Non contrôlé")</f>
         <v>Non contrôlé</v>
       </c>
-      <c r="O37" s="204"/>
+      <c r="O37" s="255"/>
       <c r="P37" s="87">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -6438,7 +6438,7 @@
       </c>
       <c r="R37" s="92"/>
       <c r="S37" s="74"/>
-      <c r="U37" s="280" t="s">
+      <c r="U37" s="195" t="s">
         <v>42</v>
       </c>
     </row>
@@ -6448,23 +6448,23 @@
       <c r="D38" s="90">
         <v>5</v>
       </c>
-      <c r="E38" s="200" t="str">
+      <c r="E38" s="251" t="str">
         <f>IFERROR(HLOOKUP($D$32,Critères!$B$3:$BE$16,D38+2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="F38" s="201"/>
-      <c r="G38" s="201"/>
-      <c r="H38" s="201"/>
-      <c r="I38" s="202"/>
-      <c r="J38" s="200" t="str">
+      <c r="F38" s="252"/>
+      <c r="G38" s="252"/>
+      <c r="H38" s="252"/>
+      <c r="I38" s="253"/>
+      <c r="J38" s="251" t="str">
         <f>IFERROR(IF(INDEX(Critères!$B$3:$BE$16, D38+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)="", "", INDEX(Critères!$B$3:$BE$16, D38+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)), "")</f>
         <v/>
       </c>
-      <c r="K38" s="201"/>
-      <c r="L38" s="201"/>
-      <c r="M38" s="202"/>
-      <c r="N38" s="203"/>
-      <c r="O38" s="204"/>
+      <c r="K38" s="252"/>
+      <c r="L38" s="252"/>
+      <c r="M38" s="253"/>
+      <c r="N38" s="254"/>
+      <c r="O38" s="255"/>
       <c r="P38" s="87">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -6475,7 +6475,7 @@
       </c>
       <c r="R38" s="92"/>
       <c r="S38" s="74"/>
-      <c r="U38" s="280" t="s">
+      <c r="U38" s="195" t="s">
         <v>41</v>
       </c>
     </row>
@@ -6485,23 +6485,23 @@
       <c r="D39" s="90">
         <v>6</v>
       </c>
-      <c r="E39" s="200" t="str">
+      <c r="E39" s="251" t="str">
         <f>IFERROR(HLOOKUP($D$32,Critères!$B$3:$BE$16,D39+2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="F39" s="201"/>
-      <c r="G39" s="201"/>
-      <c r="H39" s="201"/>
-      <c r="I39" s="202"/>
-      <c r="J39" s="200" t="str">
+      <c r="F39" s="252"/>
+      <c r="G39" s="252"/>
+      <c r="H39" s="252"/>
+      <c r="I39" s="253"/>
+      <c r="J39" s="251" t="str">
         <f>IFERROR(IF(INDEX(Critères!$B$3:$BE$16, D39+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)="", "", INDEX(Critères!$B$3:$BE$16, D39+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)), "")</f>
         <v/>
       </c>
-      <c r="K39" s="201"/>
-      <c r="L39" s="201"/>
-      <c r="M39" s="202"/>
-      <c r="N39" s="203"/>
-      <c r="O39" s="204"/>
+      <c r="K39" s="252"/>
+      <c r="L39" s="252"/>
+      <c r="M39" s="253"/>
+      <c r="N39" s="254"/>
+      <c r="O39" s="255"/>
       <c r="P39" s="87">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -6512,7 +6512,7 @@
       </c>
       <c r="R39" s="92"/>
       <c r="S39" s="74"/>
-      <c r="U39" s="280" t="s">
+      <c r="U39" s="195" t="s">
         <v>41</v>
       </c>
     </row>
@@ -6522,23 +6522,23 @@
       <c r="D40" s="90">
         <v>7</v>
       </c>
-      <c r="E40" s="200" t="str">
+      <c r="E40" s="251" t="str">
         <f>IFERROR(HLOOKUP($D$32,Critères!$B$3:$BE$16,D40+2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="F40" s="201"/>
-      <c r="G40" s="201"/>
-      <c r="H40" s="201"/>
-      <c r="I40" s="202"/>
-      <c r="J40" s="200" t="str">
+      <c r="F40" s="252"/>
+      <c r="G40" s="252"/>
+      <c r="H40" s="252"/>
+      <c r="I40" s="253"/>
+      <c r="J40" s="251" t="str">
         <f>IFERROR(IF(INDEX(Critères!$B$3:$BE$16, D40+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)="", "", INDEX(Critères!$B$3:$BE$16, D40+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)), "")</f>
         <v/>
       </c>
-      <c r="K40" s="201"/>
-      <c r="L40" s="201"/>
-      <c r="M40" s="202"/>
-      <c r="N40" s="203"/>
-      <c r="O40" s="204"/>
+      <c r="K40" s="252"/>
+      <c r="L40" s="252"/>
+      <c r="M40" s="253"/>
+      <c r="N40" s="254"/>
+      <c r="O40" s="255"/>
       <c r="P40" s="87">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -6549,7 +6549,7 @@
       </c>
       <c r="R40" s="92"/>
       <c r="S40" s="74"/>
-      <c r="U40" s="280" t="s">
+      <c r="U40" s="195" t="s">
         <v>41</v>
       </c>
     </row>
@@ -6559,23 +6559,23 @@
       <c r="D41" s="90">
         <v>8</v>
       </c>
-      <c r="E41" s="200" t="str">
+      <c r="E41" s="251" t="str">
         <f>IFERROR(HLOOKUP($D$32,Critères!$B$3:$BE$16,D41+2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="F41" s="201"/>
-      <c r="G41" s="201"/>
-      <c r="H41" s="201"/>
-      <c r="I41" s="202"/>
-      <c r="J41" s="200" t="str">
+      <c r="F41" s="252"/>
+      <c r="G41" s="252"/>
+      <c r="H41" s="252"/>
+      <c r="I41" s="253"/>
+      <c r="J41" s="251" t="str">
         <f>IFERROR(IF(INDEX(Critères!$B$3:$BE$16, D41+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)="", "", INDEX(Critères!$B$3:$BE$16, D41+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)), "")</f>
         <v/>
       </c>
-      <c r="K41" s="201"/>
-      <c r="L41" s="201"/>
-      <c r="M41" s="202"/>
-      <c r="N41" s="203"/>
-      <c r="O41" s="204"/>
+      <c r="K41" s="252"/>
+      <c r="L41" s="252"/>
+      <c r="M41" s="253"/>
+      <c r="N41" s="254"/>
+      <c r="O41" s="255"/>
       <c r="P41" s="87">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -6586,7 +6586,7 @@
       </c>
       <c r="R41" s="92"/>
       <c r="S41" s="74"/>
-      <c r="U41" s="280" t="s">
+      <c r="U41" s="195" t="s">
         <v>41</v>
       </c>
     </row>
@@ -6596,23 +6596,23 @@
       <c r="D42" s="90">
         <v>9</v>
       </c>
-      <c r="E42" s="200" t="str">
+      <c r="E42" s="251" t="str">
         <f>IFERROR(HLOOKUP($D$32,Critères!$B$3:$BE$16,D42+2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="F42" s="201"/>
-      <c r="G42" s="201"/>
-      <c r="H42" s="201"/>
-      <c r="I42" s="202"/>
-      <c r="J42" s="200" t="str">
+      <c r="F42" s="252"/>
+      <c r="G42" s="252"/>
+      <c r="H42" s="252"/>
+      <c r="I42" s="253"/>
+      <c r="J42" s="251" t="str">
         <f>IFERROR(IF(INDEX(Critères!$B$3:$BE$16, D42+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)="", "", INDEX(Critères!$B$3:$BE$16, D42+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)), "")</f>
         <v/>
       </c>
-      <c r="K42" s="201"/>
-      <c r="L42" s="201"/>
-      <c r="M42" s="202"/>
-      <c r="N42" s="203"/>
-      <c r="O42" s="204"/>
+      <c r="K42" s="252"/>
+      <c r="L42" s="252"/>
+      <c r="M42" s="253"/>
+      <c r="N42" s="254"/>
+      <c r="O42" s="255"/>
       <c r="P42" s="87">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -6623,7 +6623,7 @@
       </c>
       <c r="R42" s="92"/>
       <c r="S42" s="74"/>
-      <c r="U42" s="280" t="s">
+      <c r="U42" s="195" t="s">
         <v>39</v>
       </c>
     </row>
@@ -6633,23 +6633,23 @@
       <c r="D43" s="90">
         <v>10</v>
       </c>
-      <c r="E43" s="200" t="str">
+      <c r="E43" s="251" t="str">
         <f>IFERROR(HLOOKUP($D$32,Critères!$B$3:$BE$16,D43+2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="F43" s="201"/>
-      <c r="G43" s="201"/>
-      <c r="H43" s="201"/>
-      <c r="I43" s="202"/>
-      <c r="J43" s="200" t="str">
+      <c r="F43" s="252"/>
+      <c r="G43" s="252"/>
+      <c r="H43" s="252"/>
+      <c r="I43" s="253"/>
+      <c r="J43" s="251" t="str">
         <f>IFERROR(IF(INDEX(Critères!$B$3:$BE$16, D43+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)="", "", INDEX(Critères!$B$3:$BE$16, D43+2, MATCH($D$32, Critères!$B$3:$BE$3, 0) + 1)), "")</f>
         <v/>
       </c>
-      <c r="K43" s="201"/>
-      <c r="L43" s="201"/>
-      <c r="M43" s="202"/>
-      <c r="N43" s="203"/>
-      <c r="O43" s="204"/>
+      <c r="K43" s="252"/>
+      <c r="L43" s="252"/>
+      <c r="M43" s="253"/>
+      <c r="N43" s="254"/>
+      <c r="O43" s="255"/>
       <c r="P43" s="87">
         <f t="shared" ref="P43" si="1">IF(OR(N43="Validé",N43="Validé avec réserve"),Q43,0)</f>
         <v>0</v>
@@ -6660,57 +6660,57 @@
       </c>
       <c r="R43" s="92"/>
       <c r="S43" s="74"/>
-      <c r="U43" s="280">
+      <c r="U43" s="195">
         <v>0</v>
       </c>
     </row>
     <row r="44" spans="2:21" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B44" s="72"/>
       <c r="C44" s="91"/>
-      <c r="D44" s="205" t="s">
+      <c r="D44" s="268" t="s">
         <v>7</v>
       </c>
-      <c r="E44" s="206"/>
-      <c r="F44" s="206"/>
-      <c r="G44" s="206"/>
-      <c r="H44" s="206"/>
-      <c r="I44" s="206"/>
-      <c r="J44" s="206"/>
-      <c r="K44" s="206"/>
-      <c r="L44" s="206"/>
-      <c r="M44" s="207"/>
-      <c r="N44" s="208"/>
-      <c r="O44" s="208"/>
-      <c r="P44" s="208" t="s">
+      <c r="E44" s="269"/>
+      <c r="F44" s="269"/>
+      <c r="G44" s="269"/>
+      <c r="H44" s="269"/>
+      <c r="I44" s="269"/>
+      <c r="J44" s="269"/>
+      <c r="K44" s="269"/>
+      <c r="L44" s="269"/>
+      <c r="M44" s="270"/>
+      <c r="N44" s="271"/>
+      <c r="O44" s="271"/>
+      <c r="P44" s="271" t="s">
         <v>6</v>
       </c>
-      <c r="Q44" s="208"/>
+      <c r="Q44" s="271"/>
       <c r="R44" s="92"/>
       <c r="S44" s="74"/>
     </row>
     <row r="45" spans="2:21" ht="99.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B45" s="72"/>
       <c r="C45" s="91"/>
-      <c r="D45" s="194"/>
-      <c r="E45" s="195"/>
-      <c r="F45" s="195"/>
-      <c r="G45" s="195"/>
-      <c r="H45" s="195"/>
-      <c r="I45" s="195"/>
-      <c r="J45" s="195"/>
-      <c r="K45" s="195"/>
-      <c r="L45" s="195"/>
-      <c r="M45" s="196"/>
-      <c r="N45" s="197" t="str">
+      <c r="D45" s="262"/>
+      <c r="E45" s="263"/>
+      <c r="F45" s="263"/>
+      <c r="G45" s="263"/>
+      <c r="H45" s="263"/>
+      <c r="I45" s="263"/>
+      <c r="J45" s="263"/>
+      <c r="K45" s="263"/>
+      <c r="L45" s="263"/>
+      <c r="M45" s="264"/>
+      <c r="N45" s="265" t="str">
         <f>IF(P45&gt;80,"Validé",IF(P45&lt;70,"Non Validé", "Réserve"))</f>
         <v>Non Validé</v>
       </c>
-      <c r="O45" s="197"/>
-      <c r="P45" s="198">
+      <c r="O45" s="265"/>
+      <c r="P45" s="266">
         <f>IF(SUM(P34:P43)&gt;100,100,SUM(P34:P43))</f>
         <v>0</v>
       </c>
-      <c r="Q45" s="199"/>
+      <c r="Q45" s="267"/>
       <c r="R45" s="92"/>
       <c r="S45" s="74"/>
     </row>
@@ -6756,126 +6756,126 @@
     </row>
     <row r="48" spans="2:21" ht="20.100000000000001" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B48" s="75"/>
-      <c r="C48" s="209" t="s">
-        <v>247</v>
-      </c>
-      <c r="D48" s="210"/>
-      <c r="E48" s="210"/>
-      <c r="F48" s="210"/>
-      <c r="G48" s="210"/>
-      <c r="H48" s="210"/>
-      <c r="I48" s="210"/>
-      <c r="J48" s="210"/>
-      <c r="K48" s="210"/>
-      <c r="L48" s="210"/>
-      <c r="M48" s="210"/>
-      <c r="N48" s="210"/>
-      <c r="O48" s="210"/>
-      <c r="P48" s="210"/>
-      <c r="Q48" s="210"/>
-      <c r="R48" s="211"/>
+      <c r="C48" s="211" t="s">
+        <v>246</v>
+      </c>
+      <c r="D48" s="212"/>
+      <c r="E48" s="212"/>
+      <c r="F48" s="212"/>
+      <c r="G48" s="212"/>
+      <c r="H48" s="212"/>
+      <c r="I48" s="212"/>
+      <c r="J48" s="212"/>
+      <c r="K48" s="212"/>
+      <c r="L48" s="212"/>
+      <c r="M48" s="212"/>
+      <c r="N48" s="212"/>
+      <c r="O48" s="212"/>
+      <c r="P48" s="212"/>
+      <c r="Q48" s="212"/>
+      <c r="R48" s="213"/>
       <c r="S48" s="77"/>
     </row>
     <row r="49" spans="2:19" ht="20.100000000000001" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
       <c r="B49" s="75"/>
-      <c r="C49" s="246" t="s">
+      <c r="C49" s="214" t="s">
         <v>191</v>
       </c>
-      <c r="D49" s="247"/>
-      <c r="E49" s="247"/>
-      <c r="F49" s="247"/>
-      <c r="G49" s="247"/>
-      <c r="H49" s="247"/>
-      <c r="I49" s="247"/>
-      <c r="J49" s="247"/>
-      <c r="K49" s="247"/>
-      <c r="L49" s="247"/>
-      <c r="M49" s="247"/>
-      <c r="N49" s="247"/>
-      <c r="O49" s="247"/>
-      <c r="P49" s="247"/>
-      <c r="Q49" s="247"/>
-      <c r="R49" s="248"/>
+      <c r="D49" s="215"/>
+      <c r="E49" s="215"/>
+      <c r="F49" s="215"/>
+      <c r="G49" s="215"/>
+      <c r="H49" s="215"/>
+      <c r="I49" s="215"/>
+      <c r="J49" s="215"/>
+      <c r="K49" s="215"/>
+      <c r="L49" s="215"/>
+      <c r="M49" s="215"/>
+      <c r="N49" s="215"/>
+      <c r="O49" s="215"/>
+      <c r="P49" s="215"/>
+      <c r="Q49" s="215"/>
+      <c r="R49" s="216"/>
       <c r="S49" s="77"/>
     </row>
     <row r="50" spans="2:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B50" s="75"/>
-      <c r="C50" s="246"/>
-      <c r="D50" s="247"/>
-      <c r="E50" s="247"/>
-      <c r="F50" s="247"/>
-      <c r="G50" s="247"/>
-      <c r="H50" s="247"/>
-      <c r="I50" s="247"/>
-      <c r="J50" s="247"/>
-      <c r="K50" s="247"/>
-      <c r="L50" s="247"/>
-      <c r="M50" s="247"/>
-      <c r="N50" s="247"/>
-      <c r="O50" s="247"/>
-      <c r="P50" s="247"/>
-      <c r="Q50" s="247"/>
-      <c r="R50" s="248"/>
+      <c r="C50" s="214"/>
+      <c r="D50" s="215"/>
+      <c r="E50" s="215"/>
+      <c r="F50" s="215"/>
+      <c r="G50" s="215"/>
+      <c r="H50" s="215"/>
+      <c r="I50" s="215"/>
+      <c r="J50" s="215"/>
+      <c r="K50" s="215"/>
+      <c r="L50" s="215"/>
+      <c r="M50" s="215"/>
+      <c r="N50" s="215"/>
+      <c r="O50" s="215"/>
+      <c r="P50" s="215"/>
+      <c r="Q50" s="215"/>
+      <c r="R50" s="216"/>
       <c r="S50" s="77"/>
     </row>
     <row r="51" spans="2:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B51" s="75"/>
-      <c r="C51" s="246"/>
-      <c r="D51" s="247"/>
-      <c r="E51" s="247"/>
-      <c r="F51" s="247"/>
-      <c r="G51" s="247"/>
-      <c r="H51" s="247"/>
-      <c r="I51" s="247"/>
-      <c r="J51" s="247"/>
-      <c r="K51" s="247"/>
-      <c r="L51" s="247"/>
-      <c r="M51" s="247"/>
-      <c r="N51" s="247"/>
-      <c r="O51" s="247"/>
-      <c r="P51" s="247"/>
-      <c r="Q51" s="247"/>
-      <c r="R51" s="248"/>
+      <c r="C51" s="214"/>
+      <c r="D51" s="215"/>
+      <c r="E51" s="215"/>
+      <c r="F51" s="215"/>
+      <c r="G51" s="215"/>
+      <c r="H51" s="215"/>
+      <c r="I51" s="215"/>
+      <c r="J51" s="215"/>
+      <c r="K51" s="215"/>
+      <c r="L51" s="215"/>
+      <c r="M51" s="215"/>
+      <c r="N51" s="215"/>
+      <c r="O51" s="215"/>
+      <c r="P51" s="215"/>
+      <c r="Q51" s="215"/>
+      <c r="R51" s="216"/>
       <c r="S51" s="77"/>
     </row>
     <row r="52" spans="2:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B52" s="75"/>
-      <c r="C52" s="246"/>
-      <c r="D52" s="247"/>
-      <c r="E52" s="247"/>
-      <c r="F52" s="247"/>
-      <c r="G52" s="247"/>
-      <c r="H52" s="247"/>
-      <c r="I52" s="247"/>
-      <c r="J52" s="247"/>
-      <c r="K52" s="247"/>
-      <c r="L52" s="247"/>
-      <c r="M52" s="247"/>
-      <c r="N52" s="247"/>
-      <c r="O52" s="247"/>
-      <c r="P52" s="247"/>
-      <c r="Q52" s="247"/>
-      <c r="R52" s="248"/>
+      <c r="C52" s="214"/>
+      <c r="D52" s="215"/>
+      <c r="E52" s="215"/>
+      <c r="F52" s="215"/>
+      <c r="G52" s="215"/>
+      <c r="H52" s="215"/>
+      <c r="I52" s="215"/>
+      <c r="J52" s="215"/>
+      <c r="K52" s="215"/>
+      <c r="L52" s="215"/>
+      <c r="M52" s="215"/>
+      <c r="N52" s="215"/>
+      <c r="O52" s="215"/>
+      <c r="P52" s="215"/>
+      <c r="Q52" s="215"/>
+      <c r="R52" s="216"/>
       <c r="S52" s="77"/>
     </row>
     <row r="53" spans="2:19" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B53" s="75"/>
-      <c r="C53" s="249"/>
-      <c r="D53" s="250"/>
-      <c r="E53" s="250"/>
-      <c r="F53" s="250"/>
-      <c r="G53" s="250"/>
-      <c r="H53" s="250"/>
-      <c r="I53" s="250"/>
-      <c r="J53" s="250"/>
-      <c r="K53" s="250"/>
-      <c r="L53" s="250"/>
-      <c r="M53" s="250"/>
-      <c r="N53" s="250"/>
-      <c r="O53" s="250"/>
-      <c r="P53" s="250"/>
-      <c r="Q53" s="250"/>
-      <c r="R53" s="251"/>
+      <c r="C53" s="217"/>
+      <c r="D53" s="218"/>
+      <c r="E53" s="218"/>
+      <c r="F53" s="218"/>
+      <c r="G53" s="218"/>
+      <c r="H53" s="218"/>
+      <c r="I53" s="218"/>
+      <c r="J53" s="218"/>
+      <c r="K53" s="218"/>
+      <c r="L53" s="218"/>
+      <c r="M53" s="218"/>
+      <c r="N53" s="218"/>
+      <c r="O53" s="218"/>
+      <c r="P53" s="218"/>
+      <c r="Q53" s="218"/>
+      <c r="R53" s="219"/>
       <c r="S53" s="77"/>
     </row>
     <row r="54" spans="2:19" ht="9.9499999999999993" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
@@ -6899,33 +6899,82 @@
       <c r="S54" s="80"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="FPAlo9oZwMO5xXgttkVL284nB8BU49V8z/8Bn2eekUPqwAX4P0QQQE6XxzcU7EogpnmWJP2Tse4cy+YgSdbYFQ==" saltValue="y5qzpFlAXYZ3qiJdFGbA6A==" spinCount="100000" sheet="1" objects="1" scenarios="1" formatRows="0"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="MF5mTCx3SCqkg8qQ0hmHNPoLHL76/t1wvOtYZ7kDkhTQU6iOkgW80nPnHdJK39e7T/zYsNPg/pi6VMlLRyHFHA==" saltValue="EFGpiul+RDeLlun+OhRsTg==" spinCount="100000" sheet="1" objects="1" scenarios="1" formatRows="0"/>
   <mergeCells count="123">
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="M4:O4"/>
-    <mergeCell ref="P4:R4"/>
-    <mergeCell ref="C2:R2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J3:L3"/>
-    <mergeCell ref="M3:O3"/>
-    <mergeCell ref="P3:R3"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="M6:O6"/>
-    <mergeCell ref="P6:R6"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="M5:O5"/>
-    <mergeCell ref="P5:R5"/>
+    <mergeCell ref="D45:M45"/>
+    <mergeCell ref="N45:O45"/>
+    <mergeCell ref="P45:Q45"/>
+    <mergeCell ref="E43:I43"/>
+    <mergeCell ref="J43:M43"/>
+    <mergeCell ref="N43:O43"/>
+    <mergeCell ref="D44:M44"/>
+    <mergeCell ref="N44:O44"/>
+    <mergeCell ref="P44:Q44"/>
+    <mergeCell ref="E41:I41"/>
+    <mergeCell ref="J41:M41"/>
+    <mergeCell ref="N41:O41"/>
+    <mergeCell ref="E42:I42"/>
+    <mergeCell ref="J42:M42"/>
+    <mergeCell ref="N42:O42"/>
+    <mergeCell ref="E39:I39"/>
+    <mergeCell ref="J39:M39"/>
+    <mergeCell ref="N39:O39"/>
+    <mergeCell ref="E40:I40"/>
+    <mergeCell ref="J40:M40"/>
+    <mergeCell ref="N40:O40"/>
+    <mergeCell ref="E37:I37"/>
+    <mergeCell ref="J37:M37"/>
+    <mergeCell ref="N37:O37"/>
+    <mergeCell ref="E38:I38"/>
+    <mergeCell ref="J38:M38"/>
+    <mergeCell ref="N38:O38"/>
+    <mergeCell ref="E35:I35"/>
+    <mergeCell ref="J35:M35"/>
+    <mergeCell ref="N35:O35"/>
+    <mergeCell ref="E36:I36"/>
+    <mergeCell ref="J36:M36"/>
+    <mergeCell ref="N36:O36"/>
+    <mergeCell ref="C30:R30"/>
+    <mergeCell ref="D32:Q32"/>
+    <mergeCell ref="D33:I33"/>
+    <mergeCell ref="J33:M33"/>
+    <mergeCell ref="N33:O33"/>
+    <mergeCell ref="E34:I34"/>
+    <mergeCell ref="J34:M34"/>
+    <mergeCell ref="N34:O34"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="K25:M25"/>
+    <mergeCell ref="N25:P25"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="G22:J22"/>
+    <mergeCell ref="K21:M21"/>
+    <mergeCell ref="N21:Q21"/>
+    <mergeCell ref="K22:M22"/>
+    <mergeCell ref="N22:Q22"/>
+    <mergeCell ref="D24:M24"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="K19:M19"/>
+    <mergeCell ref="N19:Q19"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="K20:M20"/>
+    <mergeCell ref="N20:Q20"/>
+    <mergeCell ref="D17:Q17"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="K18:M18"/>
+    <mergeCell ref="N18:Q18"/>
     <mergeCell ref="C8:R8"/>
     <mergeCell ref="C48:R48"/>
     <mergeCell ref="C49:R53"/>
@@ -6950,80 +6999,31 @@
     <mergeCell ref="G13:J13"/>
     <mergeCell ref="K13:M13"/>
     <mergeCell ref="N13:Q13"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="K19:M19"/>
-    <mergeCell ref="N19:Q19"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="K20:M20"/>
-    <mergeCell ref="N20:Q20"/>
-    <mergeCell ref="D17:Q17"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="K18:M18"/>
-    <mergeCell ref="N18:Q18"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="G27:H27"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="K25:M25"/>
-    <mergeCell ref="N25:P25"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="G22:J22"/>
-    <mergeCell ref="K21:M21"/>
-    <mergeCell ref="N21:Q21"/>
-    <mergeCell ref="K22:M22"/>
-    <mergeCell ref="N22:Q22"/>
-    <mergeCell ref="D24:M24"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="C30:R30"/>
-    <mergeCell ref="D32:Q32"/>
-    <mergeCell ref="D33:I33"/>
-    <mergeCell ref="J33:M33"/>
-    <mergeCell ref="N33:O33"/>
-    <mergeCell ref="E34:I34"/>
-    <mergeCell ref="J34:M34"/>
-    <mergeCell ref="N34:O34"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="E37:I37"/>
-    <mergeCell ref="J37:M37"/>
-    <mergeCell ref="N37:O37"/>
-    <mergeCell ref="E38:I38"/>
-    <mergeCell ref="J38:M38"/>
-    <mergeCell ref="N38:O38"/>
-    <mergeCell ref="E35:I35"/>
-    <mergeCell ref="J35:M35"/>
-    <mergeCell ref="N35:O35"/>
-    <mergeCell ref="E36:I36"/>
-    <mergeCell ref="J36:M36"/>
-    <mergeCell ref="N36:O36"/>
-    <mergeCell ref="E41:I41"/>
-    <mergeCell ref="J41:M41"/>
-    <mergeCell ref="N41:O41"/>
-    <mergeCell ref="E42:I42"/>
-    <mergeCell ref="J42:M42"/>
-    <mergeCell ref="N42:O42"/>
-    <mergeCell ref="E39:I39"/>
-    <mergeCell ref="J39:M39"/>
-    <mergeCell ref="N39:O39"/>
-    <mergeCell ref="E40:I40"/>
-    <mergeCell ref="J40:M40"/>
-    <mergeCell ref="N40:O40"/>
-    <mergeCell ref="D45:M45"/>
-    <mergeCell ref="N45:O45"/>
-    <mergeCell ref="P45:Q45"/>
-    <mergeCell ref="E43:I43"/>
-    <mergeCell ref="J43:M43"/>
-    <mergeCell ref="N43:O43"/>
-    <mergeCell ref="D44:M44"/>
-    <mergeCell ref="N44:O44"/>
-    <mergeCell ref="P44:Q44"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="M6:O6"/>
+    <mergeCell ref="P6:R6"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="M5:O5"/>
+    <mergeCell ref="P5:R5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="M4:O4"/>
+    <mergeCell ref="P4:R4"/>
+    <mergeCell ref="C2:R2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:L3"/>
+    <mergeCell ref="M3:O3"/>
+    <mergeCell ref="P3:R3"/>
   </mergeCells>
   <conditionalFormatting sqref="M27">
     <cfRule type="expression" dxfId="13" priority="13">
@@ -7747,7 +7747,7 @@
       <c r="BD2" s="181"/>
       <c r="BE2" s="181"/>
       <c r="BF2" s="182" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="BG2" s="183"/>
       <c r="BH2" s="183"/>
@@ -7761,7 +7761,7 @@
       <c r="BP2" s="183"/>
       <c r="BQ2" s="183"/>
       <c r="BR2" s="184" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="BS2" s="185"/>
       <c r="BT2" s="185"/>
@@ -7819,7 +7819,7 @@
       <c r="H3" s="28"/>
       <c r="I3" s="29"/>
       <c r="J3" s="27" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="K3" s="27"/>
       <c r="L3" s="28"/>
@@ -7831,7 +7831,7 @@
       <c r="P3" s="28"/>
       <c r="Q3" s="29"/>
       <c r="R3" s="27" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="S3" s="27"/>
       <c r="T3" s="28"/>
@@ -7855,7 +7855,7 @@
       <c r="AF3" s="33"/>
       <c r="AG3" s="34"/>
       <c r="AH3" s="31" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="AI3" s="32"/>
       <c r="AJ3" s="33"/>
@@ -8160,7 +8160,7 @@
         <v>118</v>
       </c>
       <c r="C5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D5" s="125">
         <v>10</v>
@@ -8172,7 +8172,7 @@
         <v>118</v>
       </c>
       <c r="G5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H5" s="125">
         <v>10</v>
@@ -8184,7 +8184,7 @@
         <v>118</v>
       </c>
       <c r="K5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="L5" s="125">
         <v>10</v>
@@ -8196,7 +8196,7 @@
         <v>118</v>
       </c>
       <c r="O5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="P5" s="125">
         <v>10</v>
@@ -8208,7 +8208,7 @@
         <v>118</v>
       </c>
       <c r="S5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="T5" s="125">
         <v>10</v>
@@ -8220,7 +8220,7 @@
         <v>118</v>
       </c>
       <c r="W5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="X5" s="125">
         <v>10</v>
@@ -8232,7 +8232,7 @@
         <v>118</v>
       </c>
       <c r="AA5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="AB5" s="125">
         <v>10</v>
@@ -8244,7 +8244,7 @@
         <v>118</v>
       </c>
       <c r="AE5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="AF5" s="125">
         <v>10</v>
@@ -8256,7 +8256,7 @@
         <v>118</v>
       </c>
       <c r="AI5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="AJ5" s="125">
         <v>10</v>
@@ -8268,7 +8268,7 @@
         <v>118</v>
       </c>
       <c r="AM5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="AN5" s="125">
         <v>10</v>
@@ -8280,7 +8280,7 @@
         <v>118</v>
       </c>
       <c r="AQ5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="AR5" s="125">
         <v>10</v>
@@ -8292,7 +8292,7 @@
         <v>118</v>
       </c>
       <c r="AU5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="AV5" s="125">
         <v>10</v>
@@ -8304,7 +8304,7 @@
         <v>118</v>
       </c>
       <c r="AY5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="AZ5" s="125">
         <v>10</v>
@@ -8316,7 +8316,7 @@
         <v>118</v>
       </c>
       <c r="BC5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="BD5" s="125">
         <v>10</v>
@@ -8328,7 +8328,7 @@
         <v>118</v>
       </c>
       <c r="BG5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="BH5" s="125">
         <v>10</v>
@@ -8340,7 +8340,7 @@
         <v>118</v>
       </c>
       <c r="BK5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="BL5" s="125">
         <v>10</v>
@@ -8352,7 +8352,7 @@
         <v>118</v>
       </c>
       <c r="BO5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="BP5" s="125">
         <v>10</v>
@@ -8364,7 +8364,7 @@
         <v>118</v>
       </c>
       <c r="BS5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="BT5" s="125">
         <v>10</v>
@@ -8376,7 +8376,7 @@
         <v>118</v>
       </c>
       <c r="BW5" s="124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="BX5" s="125">
         <v>10</v>
@@ -8393,7 +8393,7 @@
         <v>119</v>
       </c>
       <c r="C6" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D6" s="42">
         <v>10</v>
@@ -8405,7 +8405,7 @@
         <v>119</v>
       </c>
       <c r="G6" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="H6" s="42">
         <v>10</v>
@@ -8417,7 +8417,7 @@
         <v>119</v>
       </c>
       <c r="K6" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="L6" s="42">
         <v>10</v>
@@ -8429,7 +8429,7 @@
         <v>119</v>
       </c>
       <c r="O6" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="P6" s="42">
         <v>10</v>
@@ -8441,7 +8441,7 @@
         <v>119</v>
       </c>
       <c r="S6" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="T6" s="42">
         <v>10</v>
@@ -8453,7 +8453,7 @@
         <v>120</v>
       </c>
       <c r="W6" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="X6" s="42">
         <v>10</v>
@@ -8465,7 +8465,7 @@
         <v>120</v>
       </c>
       <c r="AA6" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AB6" s="42">
         <v>10</v>
@@ -8477,7 +8477,7 @@
         <v>24</v>
       </c>
       <c r="AE6" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AF6" s="42">
         <v>10</v>
@@ -8486,7 +8486,7 @@
         <v>40</v>
       </c>
       <c r="AH6" s="40" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="AI6" s="45"/>
       <c r="AJ6" s="42">
@@ -8496,7 +8496,7 @@
         <v>40</v>
       </c>
       <c r="AL6" s="40" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="AM6" s="45"/>
       <c r="AN6" s="42">
@@ -8509,7 +8509,7 @@
         <v>119</v>
       </c>
       <c r="AQ6" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AR6" s="42">
         <v>10</v>
@@ -8521,7 +8521,7 @@
         <v>121</v>
       </c>
       <c r="AU6" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AV6" s="42">
         <v>10</v>
@@ -8530,10 +8530,10 @@
         <v>40</v>
       </c>
       <c r="AX6" s="40" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="AY6" s="45" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AZ6" s="42">
         <v>10</v>
@@ -8545,7 +8545,7 @@
         <v>122</v>
       </c>
       <c r="BC6" s="45" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BD6" s="42">
         <v>20</v>
@@ -8557,7 +8557,7 @@
         <v>25</v>
       </c>
       <c r="BG6" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BH6" s="42">
         <v>15</v>
@@ -8579,7 +8579,7 @@
         <v>27</v>
       </c>
       <c r="BO6" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BP6" s="42">
         <v>20</v>
@@ -8620,7 +8620,7 @@
         <v>123</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D7" s="132">
         <v>10</v>
@@ -8632,7 +8632,7 @@
         <v>123</v>
       </c>
       <c r="G7" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="H7" s="132">
         <v>10</v>
@@ -8644,7 +8644,7 @@
         <v>123</v>
       </c>
       <c r="K7" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="L7" s="132">
         <v>10</v>
@@ -8656,7 +8656,7 @@
         <v>123</v>
       </c>
       <c r="O7" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="P7" s="132">
         <v>10</v>
@@ -8668,7 +8668,7 @@
         <v>123</v>
       </c>
       <c r="S7" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="T7" s="132">
         <v>10</v>
@@ -8677,7 +8677,7 @@
         <v>40</v>
       </c>
       <c r="V7" s="10" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="W7" s="25" t="s">
         <v>124</v>
@@ -8689,7 +8689,7 @@
         <v>40</v>
       </c>
       <c r="Z7" s="24" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="AA7" s="25" t="s">
         <v>124</v>
@@ -8701,10 +8701,10 @@
         <v>40</v>
       </c>
       <c r="AD7" s="24" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AE7" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AF7" s="132">
         <v>10</v>
@@ -8713,7 +8713,7 @@
         <v>40</v>
       </c>
       <c r="AH7" s="24" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="AI7" s="25"/>
       <c r="AJ7" s="132">
@@ -8736,7 +8736,7 @@
         <v>126</v>
       </c>
       <c r="AQ7" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AR7" s="132">
         <v>10</v>
@@ -8748,7 +8748,7 @@
         <v>127</v>
       </c>
       <c r="AU7" s="134" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AV7" s="132">
         <v>10</v>
@@ -8760,7 +8760,7 @@
         <v>128</v>
       </c>
       <c r="AY7" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AZ7" s="132">
         <v>10</v>
@@ -8772,7 +8772,7 @@
         <v>129</v>
       </c>
       <c r="BC7" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BD7" s="132">
         <v>20</v>
@@ -8808,7 +8808,7 @@
         <v>132</v>
       </c>
       <c r="BO7" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BP7" s="132">
         <v>30</v>
@@ -8832,7 +8832,7 @@
         <v>186</v>
       </c>
       <c r="BW7" s="25" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="BX7" s="132">
         <v>20</v>
@@ -9005,7 +9005,7 @@
         <v>138</v>
       </c>
       <c r="BC8" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BD8" s="42">
         <v>20</v>
@@ -9017,7 +9017,7 @@
         <v>28</v>
       </c>
       <c r="BG8" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BH8" s="42">
         <v>5</v>
@@ -9051,7 +9051,7 @@
         <v>187</v>
       </c>
       <c r="BS8" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BT8" s="42">
         <v>30</v>
@@ -9140,7 +9140,7 @@
         <v>34</v>
       </c>
       <c r="W9" s="25" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="X9" s="132">
         <v>10</v>
@@ -9152,7 +9152,7 @@
         <v>34</v>
       </c>
       <c r="AA9" s="25" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="AB9" s="132">
         <v>10</v>
@@ -9164,7 +9164,7 @@
         <v>34</v>
       </c>
       <c r="AE9" s="25" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="AF9" s="132">
         <v>10</v>
@@ -9176,7 +9176,7 @@
         <v>143</v>
       </c>
       <c r="AI9" s="25" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="AJ9" s="132">
         <v>10</v>
@@ -9188,7 +9188,7 @@
         <v>143</v>
       </c>
       <c r="AM9" s="25" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="AN9" s="132">
         <v>10</v>
@@ -9236,7 +9236,7 @@
         <v>148</v>
       </c>
       <c r="BC9" s="134" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BD9" s="132">
         <v>20</v>
@@ -9272,7 +9272,7 @@
         <v>151</v>
       </c>
       <c r="BO9" s="139" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BP9" s="140">
         <v>20</v>
@@ -9281,20 +9281,20 @@
         <v>40</v>
       </c>
       <c r="BR9" s="10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BS9" s="139" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BT9" s="140"/>
       <c r="BU9" s="166" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="BV9" s="10" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="BW9" s="139" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BX9" s="132">
         <v>30</v>
@@ -9308,10 +9308,10 @@
         <v>6</v>
       </c>
       <c r="B10" s="47" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C10" s="48" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D10" s="49">
         <v>20</v>
@@ -9320,10 +9320,10 @@
         <v>41</v>
       </c>
       <c r="F10" s="47" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="G10" s="48" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="H10" s="49">
         <v>20</v>
@@ -9332,10 +9332,10 @@
         <v>41</v>
       </c>
       <c r="J10" s="47" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="K10" s="48" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="L10" s="49">
         <v>20</v>
@@ -9344,10 +9344,10 @@
         <v>41</v>
       </c>
       <c r="N10" s="47" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="O10" s="48" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="P10" s="49">
         <v>20</v>
@@ -9356,10 +9356,10 @@
         <v>41</v>
       </c>
       <c r="R10" s="47" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="S10" s="48" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="T10" s="49">
         <v>20</v>
@@ -9371,7 +9371,7 @@
         <v>152</v>
       </c>
       <c r="W10" s="45" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="X10" s="42">
         <v>10</v>
@@ -9383,7 +9383,7 @@
         <v>153</v>
       </c>
       <c r="AA10" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AB10" s="42">
         <v>10</v>
@@ -9392,10 +9392,10 @@
         <v>40</v>
       </c>
       <c r="AD10" s="40" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="AE10" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AF10" s="42">
         <v>10</v>
@@ -9404,7 +9404,7 @@
         <v>40</v>
       </c>
       <c r="AH10" s="40" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="AI10" s="41"/>
       <c r="AJ10" s="42">
@@ -9414,7 +9414,7 @@
         <v>40</v>
       </c>
       <c r="AL10" s="40" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="AM10" s="41"/>
       <c r="AN10" s="42">
@@ -9424,10 +9424,10 @@
         <v>40</v>
       </c>
       <c r="AP10" s="44" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="AQ10" s="45" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AR10" s="42">
         <v>10</v>
@@ -9436,10 +9436,10 @@
         <v>40</v>
       </c>
       <c r="AT10" s="40" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="AU10" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AV10" s="42">
         <v>10</v>
@@ -9451,7 +9451,7 @@
         <v>154</v>
       </c>
       <c r="AY10" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AZ10" s="42">
         <v>20</v>
@@ -9463,7 +9463,7 @@
         <v>155</v>
       </c>
       <c r="BC10" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BD10" s="42">
         <v>5</v>
@@ -9484,10 +9484,10 @@
         <v>41</v>
       </c>
       <c r="BJ10" s="111" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BK10" s="41" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="BL10" s="42">
         <v>0</v>
@@ -9496,34 +9496,34 @@
         <v>40</v>
       </c>
       <c r="BN10" s="40" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BO10" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BP10" s="42"/>
       <c r="BQ10" s="167" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="BR10" s="44" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BS10" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BT10" s="42"/>
       <c r="BU10" s="43" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="BV10" s="44" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BW10" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BX10" s="42"/>
       <c r="BY10" s="167" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="11" spans="1:603" s="23" customFormat="1" ht="140.35" x14ac:dyDescent="0.4">
@@ -9531,10 +9531,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="138" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C11" s="139" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D11" s="140">
         <v>20</v>
@@ -9543,10 +9543,10 @@
         <v>41</v>
       </c>
       <c r="F11" s="138" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="G11" s="139" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="H11" s="140">
         <v>20</v>
@@ -9555,10 +9555,10 @@
         <v>41</v>
       </c>
       <c r="J11" s="138" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="K11" s="139" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="L11" s="140">
         <v>20</v>
@@ -9567,10 +9567,10 @@
         <v>41</v>
       </c>
       <c r="N11" s="138" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="O11" s="139" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="P11" s="140">
         <v>20</v>
@@ -9579,10 +9579,10 @@
         <v>41</v>
       </c>
       <c r="R11" s="138" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="S11" s="139" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="T11" s="140">
         <v>20</v>
@@ -9594,7 +9594,7 @@
         <v>157</v>
       </c>
       <c r="W11" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="X11" s="132">
         <v>10</v>
@@ -9606,7 +9606,7 @@
         <v>157</v>
       </c>
       <c r="AA11" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AB11" s="132">
         <v>10</v>
@@ -9618,7 +9618,7 @@
         <v>157</v>
       </c>
       <c r="AE11" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AF11" s="132">
         <v>10</v>
@@ -9630,7 +9630,7 @@
         <v>157</v>
       </c>
       <c r="AI11" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AJ11" s="132">
         <v>10</v>
@@ -9642,7 +9642,7 @@
         <v>157</v>
       </c>
       <c r="AM11" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AN11" s="132">
         <v>10</v>
@@ -9654,7 +9654,7 @@
         <v>157</v>
       </c>
       <c r="AQ11" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AR11" s="132">
         <v>10</v>
@@ -9663,10 +9663,10 @@
         <v>41</v>
       </c>
       <c r="AT11" s="24" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="AU11" s="134" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AV11" s="132">
         <v>15</v>
@@ -9678,7 +9678,7 @@
         <v>158</v>
       </c>
       <c r="AY11" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AZ11" s="132">
         <v>20</v>
@@ -9690,7 +9690,7 @@
         <v>159</v>
       </c>
       <c r="BC11" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BD11" s="132">
         <v>5</v>
@@ -9702,7 +9702,7 @@
         <v>156</v>
       </c>
       <c r="BG11" s="25" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="BH11" s="132">
         <v>10</v>
@@ -9711,10 +9711,10 @@
         <v>40</v>
       </c>
       <c r="BJ11" s="186" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="BK11" s="187" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="BL11" s="188">
         <v>10</v>
@@ -9723,34 +9723,34 @@
         <v>41</v>
       </c>
       <c r="BN11" s="24" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BO11" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BP11" s="132"/>
       <c r="BQ11" s="15" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="BR11" s="10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BS11" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BT11" s="132"/>
       <c r="BU11" s="168" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="BV11" s="10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BW11" s="25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BX11" s="132"/>
       <c r="BY11" s="133" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="12" spans="1:603" s="46" customFormat="1" ht="178.35" x14ac:dyDescent="0.4">
@@ -9821,7 +9821,7 @@
         <v>162</v>
       </c>
       <c r="W12" s="41" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="X12" s="42">
         <v>10</v>
@@ -9833,7 +9833,7 @@
         <v>162</v>
       </c>
       <c r="AA12" s="41" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="AB12" s="42">
         <v>10</v>
@@ -9845,7 +9845,7 @@
         <v>162</v>
       </c>
       <c r="AE12" s="41" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="AF12" s="42">
         <v>10</v>
@@ -9857,7 +9857,7 @@
         <v>162</v>
       </c>
       <c r="AI12" s="41" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="AJ12" s="42">
         <v>10</v>
@@ -9869,7 +9869,7 @@
         <v>162</v>
       </c>
       <c r="AM12" s="41" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="AN12" s="42">
         <v>10</v>
@@ -9881,7 +9881,7 @@
         <v>162</v>
       </c>
       <c r="AQ12" s="41" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="AR12" s="42">
         <v>10</v>
@@ -9890,10 +9890,10 @@
         <v>41</v>
       </c>
       <c r="AT12" s="40" t="s">
+        <v>333</v>
+      </c>
+      <c r="AU12" s="41" t="s">
         <v>334</v>
-      </c>
-      <c r="AU12" s="41" t="s">
-        <v>335</v>
       </c>
       <c r="AV12" s="42">
         <v>15</v>
@@ -9914,20 +9914,20 @@
         <v>41</v>
       </c>
       <c r="BB12" s="40" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BC12" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BD12" s="42"/>
       <c r="BE12" s="43" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="BF12" s="40" t="s">
         <v>36</v>
       </c>
       <c r="BG12" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BH12" s="42">
         <v>5</v>
@@ -9939,7 +9939,7 @@
         <v>36</v>
       </c>
       <c r="BK12" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BL12" s="42">
         <v>5</v>
@@ -9948,34 +9948,34 @@
         <v>41</v>
       </c>
       <c r="BN12" s="40" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BO12" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BP12" s="42"/>
       <c r="BQ12" s="169" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="BR12" s="44" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BS12" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BT12" s="42"/>
       <c r="BU12" s="167" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="BV12" s="44" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BW12" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BX12" s="42"/>
       <c r="BY12" s="170" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="13" spans="1:603" s="23" customFormat="1" ht="93.35" x14ac:dyDescent="0.4">
@@ -9986,7 +9986,7 @@
         <v>37</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D13" s="14">
         <v>20</v>
@@ -9998,7 +9998,7 @@
         <v>37</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="H13" s="14">
         <v>20</v>
@@ -10010,7 +10010,7 @@
         <v>37</v>
       </c>
       <c r="K13" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="L13" s="14">
         <v>20</v>
@@ -10022,7 +10022,7 @@
         <v>37</v>
       </c>
       <c r="O13" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="P13" s="14">
         <v>20</v>
@@ -10031,10 +10031,10 @@
         <v>39</v>
       </c>
       <c r="R13" s="12" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="S13" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="T13" s="14">
         <v>20</v>
@@ -10115,10 +10115,10 @@
         <v>41</v>
       </c>
       <c r="AT13" s="12" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AU13" s="13" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="AV13" s="14">
         <v>0</v>
@@ -10130,7 +10130,7 @@
         <v>169</v>
       </c>
       <c r="AY13" s="146" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AZ13" s="147">
         <v>20</v>
@@ -10139,20 +10139,20 @@
         <v>41</v>
       </c>
       <c r="BB13" s="24" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BC13" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BD13" s="14"/>
       <c r="BE13" s="15" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="BF13" s="12" t="s">
         <v>165</v>
       </c>
       <c r="BG13" s="149" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BH13" s="14">
         <v>15</v>
@@ -10164,7 +10164,7 @@
         <v>165</v>
       </c>
       <c r="BK13" s="191" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BL13" s="192">
         <v>15</v>
@@ -10173,34 +10173,34 @@
         <v>41</v>
       </c>
       <c r="BN13" s="12" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BO13" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BP13" s="14"/>
       <c r="BQ13" s="168" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="BR13" s="144" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BS13" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BT13" s="14"/>
       <c r="BU13" s="133" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="BV13" s="144" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BW13" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BX13" s="14"/>
       <c r="BY13" s="133" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="14" spans="1:603" s="46" customFormat="1" ht="38.35" thickBot="1" x14ac:dyDescent="0.45">
@@ -10208,60 +10208,60 @@
         <v>10</v>
       </c>
       <c r="B14" s="53" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D14" s="55"/>
       <c r="E14" s="56" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F14" s="53" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="G14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="H14" s="55"/>
       <c r="I14" s="56" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="J14" s="53" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="K14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="L14" s="55"/>
       <c r="M14" s="56" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="N14" s="53" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="O14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="P14" s="55"/>
       <c r="Q14" s="56" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="R14" s="53" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="S14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="T14" s="55"/>
       <c r="U14" s="56" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="V14" s="57" t="s">
         <v>168</v>
       </c>
       <c r="W14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="X14" s="55">
         <v>10</v>
@@ -10273,7 +10273,7 @@
         <v>168</v>
       </c>
       <c r="AA14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AB14" s="55">
         <v>10</v>
@@ -10285,7 +10285,7 @@
         <v>168</v>
       </c>
       <c r="AE14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AF14" s="55">
         <v>10</v>
@@ -10297,7 +10297,7 @@
         <v>168</v>
       </c>
       <c r="AI14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AJ14" s="55">
         <v>10</v>
@@ -10309,7 +10309,7 @@
         <v>168</v>
       </c>
       <c r="AM14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AN14" s="55">
         <v>10</v>
@@ -10321,7 +10321,7 @@
         <v>168</v>
       </c>
       <c r="AQ14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AR14" s="55">
         <v>10</v>
@@ -10330,22 +10330,22 @@
         <v>39</v>
       </c>
       <c r="AT14" s="53" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="AU14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AV14" s="55">
         <v>10</v>
       </c>
       <c r="AW14" s="56" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="AX14" s="53" t="s">
         <v>170</v>
       </c>
       <c r="AY14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AZ14" s="55">
         <v>10</v>
@@ -10354,20 +10354,20 @@
         <v>39</v>
       </c>
       <c r="BB14" s="53" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BC14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BD14" s="55"/>
       <c r="BE14" s="56" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="BF14" s="53" t="s">
         <v>38</v>
       </c>
       <c r="BG14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BH14" s="55">
         <v>25</v>
@@ -10379,43 +10379,43 @@
         <v>38</v>
       </c>
       <c r="BK14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BL14" s="55">
         <v>30</v>
       </c>
       <c r="BM14" s="172" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="BN14" s="53" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BO14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BP14" s="55"/>
       <c r="BQ14" s="56" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="BR14" s="57" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BS14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BT14" s="55"/>
       <c r="BU14" s="173" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="BV14" s="57" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BW14" s="54" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BX14" s="55"/>
       <c r="BY14" s="173" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="15" spans="1:603" s="11" customFormat="1" x14ac:dyDescent="0.4">
@@ -18386,10 +18386,10 @@
       <c r="H3" s="59" t="s">
         <v>45</v>
       </c>
-      <c r="I3" s="270" t="s">
-        <v>275</v>
-      </c>
-      <c r="J3" s="271"/>
+      <c r="I3" s="272" t="s">
+        <v>274</v>
+      </c>
+      <c r="J3" s="273"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
@@ -18420,7 +18420,7 @@
         <v>49</v>
       </c>
       <c r="J4" s="115" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.4">
@@ -18452,7 +18452,7 @@
         <v>46</v>
       </c>
       <c r="J5" s="115" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.4">
@@ -18478,7 +18478,7 @@
         <v>10</v>
       </c>
       <c r="J6" s="116" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.4">
@@ -18486,7 +18486,7 @@
         <v>16</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>57</v>
@@ -18498,7 +18498,7 @@
         <v>57</v>
       </c>
       <c r="J7" s="116" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.4">
@@ -18516,12 +18516,12 @@
         <v>60</v>
       </c>
       <c r="J8" s="116" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>61</v>
@@ -18534,7 +18534,7 @@
         <v>62</v>
       </c>
       <c r="J9" s="115" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.4">
@@ -18549,7 +18549,7 @@
         <v>64</v>
       </c>
       <c r="J10" s="115" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.4">
@@ -18563,7 +18563,7 @@
         <v>47</v>
       </c>
       <c r="J11" s="115" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.4">
@@ -18577,7 +18577,7 @@
         <v>56</v>
       </c>
       <c r="J12" s="115" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.4">
@@ -18591,7 +18591,7 @@
         <v>65</v>
       </c>
       <c r="J13" s="115" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.4">
@@ -18605,7 +18605,7 @@
         <v>68</v>
       </c>
       <c r="J14" s="115" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.4">
@@ -18619,7 +18619,7 @@
         <v>66</v>
       </c>
       <c r="J15" s="115" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.4">
@@ -18627,10 +18627,10 @@
         <v>50</v>
       </c>
       <c r="I16" s="117" t="s">
+        <v>286</v>
+      </c>
+      <c r="J16" s="118" t="s">
         <v>287</v>
-      </c>
-      <c r="J16" s="118" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.4">
@@ -18638,10 +18638,10 @@
         <v>52</v>
       </c>
       <c r="I17" s="117" t="s">
+        <v>288</v>
+      </c>
+      <c r="J17" s="118" t="s">
         <v>289</v>
-      </c>
-      <c r="J17" s="118" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.4">
@@ -18649,10 +18649,10 @@
         <v>64</v>
       </c>
       <c r="I18" s="117" t="s">
+        <v>290</v>
+      </c>
+      <c r="J18" s="118" t="s">
         <v>291</v>
-      </c>
-      <c r="J18" s="118" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.4">
@@ -18660,10 +18660,10 @@
         <v>71</v>
       </c>
       <c r="I19" s="117" t="s">
+        <v>292</v>
+      </c>
+      <c r="J19" s="118" t="s">
         <v>293</v>
-      </c>
-      <c r="J19" s="118" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.4">
@@ -18684,14 +18684,14 @@
         <v>42</v>
       </c>
       <c r="G20" s="58" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="117" t="s">
+        <v>294</v>
+      </c>
+      <c r="J20" s="118" t="s">
         <v>295</v>
-      </c>
-      <c r="J20" s="118" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.4">
@@ -18711,14 +18711,14 @@
         <v>48</v>
       </c>
       <c r="G21" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H21" s="1"/>
       <c r="I21" s="117" t="s">
+        <v>296</v>
+      </c>
+      <c r="J21" s="118" t="s">
         <v>297</v>
-      </c>
-      <c r="J21" s="118" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.4">
@@ -18742,12 +18742,12 @@
         <v>67</v>
       </c>
       <c r="J22" s="118" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A23" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>11</v>
@@ -18766,45 +18766,45 @@
         <v>70</v>
       </c>
       <c r="J23" s="115" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.4">
       <c r="B24" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>11</v>
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="117" t="s">
+        <v>300</v>
+      </c>
+      <c r="J24" s="118" t="s">
         <v>301</v>
-      </c>
-      <c r="J24" s="118" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="C25" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>59</v>
       </c>
       <c r="F25" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="I25" s="117" t="s">
+        <v>302</v>
+      </c>
+      <c r="J25" s="118" t="s">
         <v>303</v>
-      </c>
-      <c r="J25" s="118" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.4">
@@ -18815,18 +18815,18 @@
         <v>63</v>
       </c>
       <c r="J26" s="115" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.4">
       <c r="D27" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="I27" s="117" t="s">
+        <v>304</v>
+      </c>
+      <c r="J27" s="118" t="s">
         <v>305</v>
-      </c>
-      <c r="J27" s="118" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.4">
@@ -18835,10 +18835,10 @@
       </c>
       <c r="B28" s="58"/>
       <c r="I28" s="117" t="s">
+        <v>306</v>
+      </c>
+      <c r="J28" s="118" t="s">
         <v>307</v>
-      </c>
-      <c r="J28" s="118" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.4">
@@ -18849,19 +18849,19 @@
         <v>90</v>
       </c>
       <c r="C29" s="102" t="s">
+        <v>262</v>
+      </c>
+      <c r="D29" s="102" t="s">
         <v>263</v>
       </c>
-      <c r="D29" s="102" t="s">
-        <v>264</v>
-      </c>
       <c r="E29" s="61" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="I29" s="114" t="s">
         <v>71</v>
       </c>
       <c r="J29" s="115" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.4">
@@ -18872,10 +18872,10 @@
         <v>14</v>
       </c>
       <c r="C30" s="103" t="s">
+        <v>264</v>
+      </c>
+      <c r="D30" s="103" t="s">
         <v>265</v>
-      </c>
-      <c r="D30" s="103" t="s">
-        <v>266</v>
       </c>
       <c r="E30" s="8" t="s">
         <v>15</v>
@@ -18884,7 +18884,7 @@
         <v>50</v>
       </c>
       <c r="J30" s="119" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.4">
@@ -18895,36 +18895,36 @@
         <v>16</v>
       </c>
       <c r="C31" s="103" t="s">
+        <v>266</v>
+      </c>
+      <c r="D31" s="103" t="s">
         <v>267</v>
-      </c>
-      <c r="D31" s="103" t="s">
-        <v>268</v>
       </c>
       <c r="I31" s="114" t="s">
         <v>52</v>
       </c>
       <c r="J31" s="115" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A32" s="8" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B32" s="9" t="s">
         <v>2</v>
       </c>
       <c r="C32" s="103" t="s">
+        <v>268</v>
+      </c>
+      <c r="D32" s="103" t="s">
         <v>269</v>
-      </c>
-      <c r="D32" s="103" t="s">
-        <v>270</v>
       </c>
       <c r="I32" s="114" t="s">
         <v>55</v>
       </c>
       <c r="J32" s="115" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.4">
@@ -18932,18 +18932,18 @@
         <v>88</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="I33" s="120" t="s">
         <v>58</v>
       </c>
       <c r="J33" s="121" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A34" s="8" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B34" s="9" t="s">
         <v>18</v>
@@ -19026,7 +19026,7 @@
         <v>172</v>
       </c>
       <c r="G44" s="96" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.4">
@@ -19086,7 +19086,7 @@
         <v>108</v>
       </c>
       <c r="G47" s="96" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.4">
@@ -19114,32 +19114,32 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A53" s="97" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A54" s="98" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A55" s="64" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A58" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -19202,17 +19202,17 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="17.7" x14ac:dyDescent="0.55000000000000004">
-      <c r="B2" s="272" t="s">
-        <v>321</v>
-      </c>
-      <c r="C2" s="272"/>
-      <c r="D2" s="272"/>
-      <c r="E2" s="272"/>
-      <c r="F2" s="272"/>
-      <c r="G2" s="272"/>
-      <c r="H2" s="272"/>
-      <c r="I2" s="272"/>
-      <c r="J2" s="272"/>
+      <c r="B2" s="274" t="s">
+        <v>320</v>
+      </c>
+      <c r="C2" s="274"/>
+      <c r="D2" s="274"/>
+      <c r="E2" s="274"/>
+      <c r="F2" s="274"/>
+      <c r="G2" s="274"/>
+      <c r="H2" s="274"/>
+      <c r="I2" s="274"/>
+      <c r="J2" s="274"/>
     </row>
     <row r="3" spans="2:10" ht="15.35" x14ac:dyDescent="0.5">
       <c r="B3" s="151"/>
@@ -19226,64 +19226,64 @@
       <c r="J3" s="151"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.4">
-      <c r="B4" s="273" t="s">
+      <c r="B4" s="275" t="s">
+        <v>321</v>
+      </c>
+      <c r="C4" s="275"/>
+      <c r="D4" s="152" t="s">
         <v>322</v>
-      </c>
-      <c r="C4" s="273"/>
-      <c r="D4" s="152" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.4">
-      <c r="B6" s="273" t="s">
-        <v>324</v>
-      </c>
-      <c r="C6" s="273"/>
+      <c r="B6" s="275" t="s">
+        <v>323</v>
+      </c>
+      <c r="C6" s="275"/>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.4">
-      <c r="B8" s="274" t="s">
-        <v>325</v>
-      </c>
-      <c r="C8" s="276" t="str">
+      <c r="B8" s="276" t="s">
+        <v>324</v>
+      </c>
+      <c r="C8" s="278" t="str">
         <f>Critères!B3</f>
         <v>Débitmètre électromagnétique (Eau)</v>
       </c>
-      <c r="D8" s="277"/>
-      <c r="E8" s="277"/>
-      <c r="F8" s="278"/>
-      <c r="G8" s="276" t="str">
+      <c r="D8" s="279"/>
+      <c r="E8" s="279"/>
+      <c r="F8" s="280"/>
+      <c r="G8" s="278" t="str">
         <f>Critères!N3</f>
         <v>Débitmètre Ultrason</v>
       </c>
-      <c r="H8" s="277"/>
-      <c r="I8" s="277"/>
-      <c r="J8" s="278"/>
+      <c r="H8" s="279"/>
+      <c r="I8" s="279"/>
+      <c r="J8" s="280"/>
     </row>
     <row r="9" spans="2:10" ht="27.35" x14ac:dyDescent="0.4">
-      <c r="B9" s="275"/>
+      <c r="B9" s="277"/>
       <c r="C9" s="153" t="s">
+        <v>325</v>
+      </c>
+      <c r="D9" s="154" t="s">
         <v>326</v>
       </c>
-      <c r="D9" s="154" t="s">
+      <c r="E9" s="154" t="s">
         <v>327</v>
       </c>
-      <c r="E9" s="154" t="s">
+      <c r="F9" s="155" t="s">
         <v>328</v>
       </c>
-      <c r="F9" s="155" t="s">
-        <v>329</v>
-      </c>
       <c r="G9" s="153" t="s">
+        <v>325</v>
+      </c>
+      <c r="H9" s="154" t="s">
         <v>326</v>
       </c>
-      <c r="H9" s="154" t="s">
+      <c r="I9" s="154" t="s">
         <v>327</v>
       </c>
-      <c r="I9" s="154" t="s">
+      <c r="J9" s="155" t="s">
         <v>328</v>
-      </c>
-      <c r="J9" s="155" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.4">
@@ -20597,18 +20597,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -20631,6 +20631,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB702087-7E88-4AF3-B693-D27B95F8995C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA52DDF1-DB9E-4C0C-9E16-F265EDFF44E6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="81251141-7599-4081-9962-8622873f55aa"/>
@@ -20645,12 +20653,4 @@
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB702087-7E88-4AF3-B693-D27B95F8995C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>